<commit_message>
Add sliding window and string manipulation algorithms with excel updates
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2FC528-3711-4525-B25B-60FAF9A6FDF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D5C059-9785-4643-8839-3B0A4165D682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="112">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -388,6 +388,15 @@
   </si>
   <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t>Hard</t>
+  </si>
+  <si>
+    <t>2E-2M-1H</t>
+  </si>
+  <si>
+    <t>1E-2M-2H</t>
   </si>
 </sst>
 </file>
@@ -399,7 +408,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="dd/mmm/yyyy"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -516,8 +525,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -590,6 +612,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -619,7 +647,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -696,6 +724,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1356,14 +1392,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.03</v>
+        <v>6.6666666666666666E-2</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1372,21 +1408,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="17" x14ac:dyDescent="0.4">
@@ -1532,7 +1568,7 @@
         <v>107</v>
       </c>
       <c r="U10" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="13" t="s">
         <v>108</v>
@@ -1552,7 +1588,9 @@
       <c r="D11" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="E11" s="14"/>
+      <c r="E11" s="14">
+        <v>3</v>
+      </c>
       <c r="F11" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/move-zeroes/","Move Zeroes")</f>
         <v>Move Zeroes</v>
@@ -1597,12 +1635,18 @@
         <f>HYPERLINK("https://leetcode.com/problems/3sum/","3Sum")</f>
         <v>3Sum</v>
       </c>
-      <c r="S11" s="14"/>
+      <c r="S11" s="14" t="s">
+        <v>34</v>
+      </c>
       <c r="T11" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="U11" s="14"/>
-      <c r="V11" s="14"/>
+      <c r="U11" s="14">
+        <v>2</v>
+      </c>
+      <c r="V11" s="13" t="s">
+        <v>108</v>
+      </c>
       <c r="W11" s="17"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.35">
@@ -1616,85 +1660,147 @@
       <c r="C12" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="13"/>
-      <c r="R12" s="11"/>
-      <c r="S12" s="13"/>
-      <c r="T12" s="13"/>
-      <c r="U12" s="13"/>
-      <c r="V12" s="13"/>
+      <c r="D12" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="E12" s="13">
+        <v>3</v>
+      </c>
+      <c r="F12" s="29" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/maximum-average-subarray-i/","Maximum Average Subarray I")</f>
+        <v>Maximum Average Subarray I</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="H12" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="I12" s="29" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/contains-duplicate-ii/","Contains Duplicate II")</f>
+        <v>Contains Duplicate II</v>
+      </c>
+      <c r="J12" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="K12" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="L12" s="29" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/best-time-to-buy-and-sell-stock/","Best Time to Buy and Sell Stock")</f>
+        <v>Best Time to Buy and Sell Stock</v>
+      </c>
+      <c r="M12" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="N12" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="O12" s="29" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/find-pivot-index/","Find Pivot Index")</f>
+        <v>Find Pivot Index</v>
+      </c>
+      <c r="P12" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q12" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="R12" s="29" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/longest-substring-without-repeating-characters/","Longest Substring Without Repeating Characters")</f>
+        <v>Longest Substring Without Repeating Characters</v>
+      </c>
+      <c r="S12" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="T12" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="U12" s="13">
+        <v>2</v>
+      </c>
+      <c r="V12" s="13" t="s">
+        <v>108</v>
+      </c>
       <c r="W12" s="16"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="10">
         <v>4</v>
       </c>
-      <c r="B13" s="23">
-        <f t="shared" ref="B13" si="0">B12+1</f>
-        <v>45806</v>
-      </c>
+      <c r="B13" s="23"/>
       <c r="C13" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="14"/>
-      <c r="N13" s="14"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="14"/>
-      <c r="Q13" s="14"/>
-      <c r="R13" s="12"/>
-      <c r="S13" s="14"/>
-      <c r="T13" s="14"/>
-      <c r="U13" s="14"/>
-      <c r="V13" s="14"/>
-      <c r="W13" s="17"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="10">
         <v>5</v>
       </c>
-      <c r="B14" s="23"/>
+      <c r="B14" s="23">
+        <f>B12+1</f>
+        <v>45806</v>
+      </c>
       <c r="C14" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="13"/>
+      <c r="D14" s="13" t="s">
+        <v>42</v>
+      </c>
       <c r="E14" s="13"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="13"/>
-      <c r="R14" s="11"/>
-      <c r="S14" s="13"/>
-      <c r="T14" s="13"/>
-      <c r="U14" s="13"/>
+      <c r="F14" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/valid-palindrome/","Valid Palindrome")</f>
+        <v>Valid Palindrome</v>
+      </c>
+      <c r="G14" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="H14" s="32" t="s">
+        <v>107</v>
+      </c>
+      <c r="I14" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/reverse-string/","Reverse String")</f>
+        <v>Reverse String</v>
+      </c>
+      <c r="J14" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="K14" s="32" t="s">
+        <v>107</v>
+      </c>
+      <c r="L14" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/length-of-last-word/","Length of Last Word")</f>
+        <v>Length of Last Word</v>
+      </c>
+      <c r="M14" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="N14" s="32" t="s">
+        <v>107</v>
+      </c>
+      <c r="O14" s="33" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/reverse-words-in-a-string/","Reverse Words in a String")</f>
+        <v>Reverse Words in a String</v>
+      </c>
+      <c r="P14" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q14" s="32" t="s">
+        <v>106</v>
+      </c>
+      <c r="R14" s="33" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/shortest-palindrome/","Shortest Palindrome")</f>
+        <v>Shortest Palindrome</v>
+      </c>
+      <c r="S14" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="T14" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="U14" s="13">
+        <v>4</v>
+      </c>
       <c r="V14" s="13"/>
       <c r="W14" s="16"/>
     </row>
@@ -1706,7 +1812,9 @@
       <c r="C15" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="14"/>
+      <c r="D15" s="14" t="s">
+        <v>110</v>
+      </c>
       <c r="E15" s="14"/>
       <c r="F15" s="12"/>
       <c r="G15" s="14"/>
@@ -1735,7 +1843,9 @@
       <c r="C16" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="13"/>
+      <c r="D16" s="13" t="s">
+        <v>111</v>
+      </c>
       <c r="E16" s="13"/>
       <c r="F16" s="11"/>
       <c r="G16" s="13"/>
@@ -1848,7 +1958,7 @@
         <v>11</v>
       </c>
       <c r="B20" s="23"/>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="30" t="s">
         <v>53</v>
       </c>
       <c r="D20" s="13"/>
@@ -3340,7 +3450,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G10:G69">
+  <conditionalFormatting sqref="G10:G12 G14:G69">
     <cfRule type="containsText" dxfId="22" priority="1" operator="containsText" text="Solved">
       <formula>NOT(ISERROR(SEARCH("Solved",G10)))</formula>
     </cfRule>
@@ -3354,7 +3464,7 @@
       <formula>NOT(ISERROR(SEARCH("Skipped",G10)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J10:J69">
+  <conditionalFormatting sqref="J10:J12 J14:J69">
     <cfRule type="containsText" dxfId="18" priority="5" operator="containsText" text="Solved">
       <formula>NOT(ISERROR(SEARCH("Solved",J10)))</formula>
     </cfRule>
@@ -3368,7 +3478,7 @@
       <formula>NOT(ISERROR(SEARCH("Skipped",J10)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M10:M69">
+  <conditionalFormatting sqref="M10:M12 M14:M69">
     <cfRule type="containsText" dxfId="14" priority="9" operator="containsText" text="Solved">
       <formula>NOT(ISERROR(SEARCH("Solved",M10)))</formula>
     </cfRule>
@@ -3382,7 +3492,7 @@
       <formula>NOT(ISERROR(SEARCH("Skipped",M10)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P10:P69">
+  <conditionalFormatting sqref="P10:P12 P14:P69">
     <cfRule type="containsText" dxfId="10" priority="13" operator="containsText" text="Solved">
       <formula>NOT(ISERROR(SEARCH("Solved",P10)))</formula>
     </cfRule>
@@ -3396,7 +3506,7 @@
       <formula>NOT(ISERROR(SEARCH("Skipped",P10)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S10:S69">
+  <conditionalFormatting sqref="S10:S12 S14:S69">
     <cfRule type="containsText" dxfId="6" priority="17" operator="containsText" text="Solved">
       <formula>NOT(ISERROR(SEARCH("Solved",S10)))</formula>
     </cfRule>
@@ -3410,7 +3520,7 @@
       <formula>NOT(ISERROR(SEARCH("Skipped",S10)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V10:V69">
+  <conditionalFormatting sqref="V10:V12 V14:V69">
     <cfRule type="containsText" dxfId="2" priority="21" operator="containsText" text="Done">
       <formula>NOT(ISERROR(SEARCH("Done",V10)))</formula>
     </cfRule>
@@ -3422,20 +3532,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G10:G69 J10:J69 M10:M69 P10:P69 S10:S69" xr:uid="{E9D55A71-CD17-44C2-A5C0-197B57D54800}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J14:J69 M14:M69 P14:P69 S14:S69 S10:S12 P10:P12 M10:M12 J10:J12 G10:G12 G14:G69" xr:uid="{E9D55A71-CD17-44C2-A5C0-197B57D54800}">
       <formula1>"Solved,Partial,Stuck,Skipped"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10:H69 K10:K69 N10:N69 Q10:Q69 T10:T69" xr:uid="{CAA1AB83-869C-40C8-B4BF-ABCC46363A0C}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K14:K69 N14:N69 Q14:Q69 T14:T69 T10:T12 Q10:Q12 N10:N12 K10:K12 H10:H12 H14:H69" xr:uid="{CAA1AB83-869C-40C8-B4BF-ABCC46363A0C}">
       <formula1>"Easy,Medium,Hard"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10:D69" xr:uid="{EB8389DE-9A7E-4BE0-A0CD-E46497E667CE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10:D12 D14:D69" xr:uid="{EB8389DE-9A7E-4BE0-A0CD-E46497E667CE}">
       <formula1>"2E-2M-1H,1E-3M-1H,3E-2M,2M-3H,1E-2M-2H,All Easy,All Medium,Mock"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U10:U69" xr:uid="{94F8B5A5-4188-4E83-BA45-970C2B3977DA}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U10:U12 U14:U69" xr:uid="{94F8B5A5-4188-4E83-BA45-970C2B3977DA}">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V69" xr:uid="{3B5CC177-382D-4CF3-B586-1836A6C5F18E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V12 V14:V69" xr:uid="{3B5CC177-382D-4CF3-B586-1836A6C5F18E}">
       <formula1>"Not Started,In Progress,Done,Missed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add palindrome and anagram solutions to practice notebooks and update tracking sheet
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D5C059-9785-4643-8839-3B0A4165D682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D26D9AC-4AE9-4929-86A5-6F19C5D181DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
+    <workbookView xWindow="22932" yWindow="-1416" windowWidth="23256" windowHeight="12456" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1747,7 +1747,9 @@
       <c r="D14" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="13"/>
+      <c r="E14" s="13">
+        <v>2</v>
+      </c>
       <c r="F14" s="31" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/valid-palindrome/","Valid Palindrome")</f>
         <v>Valid Palindrome</v>
@@ -1793,7 +1795,7 @@
         <v>Shortest Palindrome</v>
       </c>
       <c r="S14" s="32" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T14" s="32" t="s">
         <v>109</v>

</xml_diff>

<commit_message>
Hashing fundamentals and frequency problems  while updating String palindrome exercises
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D26D9AC-4AE9-4929-86A5-6F19C5D181DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1597EC-5F82-455F-8EC1-64941F817800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-1416" windowWidth="23256" windowHeight="12456" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="114">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -150,9 +150,6 @@
     <t>Day Status</t>
   </si>
   <si>
-    <t>Notes / Revisit</t>
-  </si>
-  <si>
     <t>Queues &amp; Deque - Sliding Window Maximum</t>
   </si>
   <si>
@@ -397,6 +394,15 @@
   </si>
   <si>
     <t>1E-2M-2H</t>
+  </si>
+  <si>
+    <t>1E-3M-1H</t>
+  </si>
+  <si>
+    <t>LeetCode Rank</t>
+  </si>
+  <si>
+    <t>~35 Lakhs</t>
   </si>
 </sst>
 </file>
@@ -539,7 +545,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -618,6 +624,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -647,7 +659,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -720,18 +732,43 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1315,7 +1352,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="526" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1342,7 +1379,7 @@
   <cols>
     <col min="1" max="1" width="20.453125" customWidth="1"/>
     <col min="2" max="2" width="16.90625" style="22" customWidth="1"/>
-    <col min="3" max="3" width="37.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.26953125" bestFit="1" customWidth="1"/>
@@ -1357,7 +1394,7 @@
     <col min="15" max="15" width="23.36328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="7.6328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.26953125" customWidth="1"/>
+    <col min="18" max="18" width="21.26953125" customWidth="1"/>
     <col min="19" max="19" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="7.6328125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="14.90625" bestFit="1" customWidth="1"/>
@@ -1367,12 +1404,15 @@
   <sheetData>
     <row r="1" spans="1:23" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
+      </c>
+      <c r="C1" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="16" x14ac:dyDescent="0.4">
@@ -1392,14 +1432,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.11666666666666667</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1408,21 +1448,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.75</v>
+        <v>2.7142857142857144</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="17" x14ac:dyDescent="0.4">
@@ -1498,7 +1538,7 @@
         <v>28</v>
       </c>
       <c r="W9" s="24" t="s">
-        <v>29</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
@@ -1509,71 +1549,73 @@
         <v>45803</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E10" s="13">
         <v>2</v>
       </c>
-      <c r="F10" s="29" t="str">
+      <c r="F10" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/contains-duplicate/","Array contain duplicates")</f>
         <v>Array contain duplicates</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="I10" s="29" t="str">
+        <v>106</v>
+      </c>
+      <c r="I10" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/two-sum/","Two Sum")</f>
         <v>Two Sum</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="L10" s="29" t="str">
+        <v>106</v>
+      </c>
+      <c r="L10" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/missing-number/","Missing Number[0,n]")</f>
         <v>Missing Number[0,n]</v>
       </c>
       <c r="M10" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N10" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="O10" s="29" t="str">
+        <v>106</v>
+      </c>
+      <c r="O10" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/find-all-numbers-disappeared-in-an-array/","Disapperaed Numbers[1,n]")</f>
         <v>Disapperaed Numbers[1,n]</v>
       </c>
       <c r="P10" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q10" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="R10" s="29" t="str">
+        <v>106</v>
+      </c>
+      <c r="R10" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/majority-element/","Majority Element")</f>
         <v>Majority Element</v>
       </c>
       <c r="S10" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T10" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="U10" s="13">
         <v>3</v>
       </c>
       <c r="V10" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="W10" s="16"/>
+        <v>107</v>
+      </c>
+      <c r="W10" s="44" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="10">
@@ -1583,69 +1625,69 @@
         <v>45804</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E11" s="14">
         <v>3</v>
       </c>
-      <c r="F11" s="28" t="str">
+      <c r="F11" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/move-zeroes/","Move Zeroes")</f>
         <v>Move Zeroes</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="I11" s="28" t="str">
+        <v>106</v>
+      </c>
+      <c r="I11" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/squares-of-a-sorted-array/","Squares of a Sorted Array")</f>
         <v>Squares of a Sorted Array</v>
       </c>
       <c r="J11" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K11" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="L11" s="28" t="str">
+        <v>106</v>
+      </c>
+      <c r="L11" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/backspace-string-compare/","Backspace String Compare")</f>
         <v>Backspace String Compare</v>
       </c>
       <c r="M11" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N11" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="O11" s="28" t="str">
+        <v>106</v>
+      </c>
+      <c r="O11" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/sort-colors/","Sort Colors")</f>
         <v>Sort Colors</v>
       </c>
       <c r="P11" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q11" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="R11" s="28" t="str">
+        <v>105</v>
+      </c>
+      <c r="R11" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/3sum/","3Sum")</f>
         <v>3Sum</v>
       </c>
       <c r="S11" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="T11" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="U11" s="14">
         <v>2</v>
       </c>
       <c r="V11" s="13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W11" s="17"/>
     </row>
@@ -1658,69 +1700,69 @@
         <v>45805</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E12" s="13">
         <v>3</v>
       </c>
-      <c r="F12" s="29" t="str">
+      <c r="F12" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/maximum-average-subarray-i/","Maximum Average Subarray I")</f>
         <v>Maximum Average Subarray I</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="I12" s="29" t="str">
+        <v>106</v>
+      </c>
+      <c r="I12" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/contains-duplicate-ii/","Contains Duplicate II")</f>
         <v>Contains Duplicate II</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="L12" s="29" t="str">
+        <v>106</v>
+      </c>
+      <c r="L12" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/best-time-to-buy-and-sell-stock/","Best Time to Buy and Sell Stock")</f>
         <v>Best Time to Buy and Sell Stock</v>
       </c>
       <c r="M12" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N12" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="O12" s="29" t="str">
+        <v>106</v>
+      </c>
+      <c r="O12" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/find-pivot-index/","Find Pivot Index")</f>
         <v>Find Pivot Index</v>
       </c>
       <c r="P12" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q12" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="R12" s="29" t="str">
+        <v>106</v>
+      </c>
+      <c r="R12" s="28" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/longest-substring-without-repeating-characters/","Longest Substring Without Repeating Characters")</f>
         <v>Longest Substring Without Repeating Characters</v>
       </c>
       <c r="S12" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T12" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="U12" s="13">
         <v>2</v>
       </c>
       <c r="V12" s="13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W12" s="16"/>
     </row>
@@ -1730,7 +1772,7 @@
       </c>
       <c r="B13" s="23"/>
       <c r="C13" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.35">
@@ -1742,189 +1784,329 @@
         <v>45806</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E14" s="13">
         <v>2</v>
       </c>
-      <c r="F14" s="31" t="str">
+      <c r="F14" s="29" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/valid-palindrome/","Valid Palindrome")</f>
         <v>Valid Palindrome</v>
       </c>
-      <c r="G14" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="H14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="I14" s="31" t="str">
+      <c r="G14" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="H14" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="I14" s="29" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/reverse-string/","Reverse String")</f>
         <v>Reverse String</v>
       </c>
-      <c r="J14" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="K14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="L14" s="31" t="str">
+      <c r="J14" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="K14" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="L14" s="29" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/length-of-last-word/","Length of Last Word")</f>
         <v>Length of Last Word</v>
       </c>
-      <c r="M14" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="N14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="O14" s="33" t="str">
+      <c r="M14" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="N14" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="O14" s="31" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/reverse-words-in-a-string/","Reverse Words in a String")</f>
         <v>Reverse Words in a String</v>
       </c>
-      <c r="P14" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q14" s="32" t="s">
-        <v>106</v>
-      </c>
-      <c r="R14" s="33" t="str">
+      <c r="P14" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q14" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="R14" s="31" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/shortest-palindrome/","Shortest Palindrome")</f>
         <v>Shortest Palindrome</v>
       </c>
-      <c r="S14" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="T14" s="32" t="s">
-        <v>109</v>
+      <c r="S14" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="T14" s="30" t="s">
+        <v>108</v>
       </c>
       <c r="U14" s="13">
         <v>4</v>
       </c>
-      <c r="V14" s="13"/>
+      <c r="V14" s="13" t="s">
+        <v>107</v>
+      </c>
       <c r="W14" s="16"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="10">
         <v>6</v>
       </c>
-      <c r="B15" s="23"/>
+      <c r="B15" s="23">
+        <f>B14+1</f>
+        <v>45807</v>
+      </c>
       <c r="C15" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="E15" s="14"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="14"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="12"/>
-      <c r="P15" s="14"/>
-      <c r="Q15" s="14"/>
-      <c r="R15" s="12"/>
-      <c r="S15" s="14"/>
-      <c r="T15" s="14"/>
-      <c r="U15" s="14"/>
-      <c r="V15" s="14"/>
+        <v>109</v>
+      </c>
+      <c r="E15" s="14">
+        <v>3</v>
+      </c>
+      <c r="F15" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/valid-anagram/","Valid Anagram")</f>
+        <v>Valid Anagram</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="I15" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/valid-palindrome-ii/","Valid Palindrome II")</f>
+        <v>Valid Palindrome II</v>
+      </c>
+      <c r="J15" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="K15" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L15" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/group-anagrams/","Group Anagrams")</f>
+        <v>Group Anagrams</v>
+      </c>
+      <c r="M15" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="N15" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="O15" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/longest-palindromic-substring/","Longest Palindromic Substring")</f>
+        <v>Longest Palindromic Substring</v>
+      </c>
+      <c r="P15" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q15" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="R15" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/palindrome-pairs/","Palindrome Pairs")</f>
+        <v>Palindrome Pairs</v>
+      </c>
+      <c r="S15" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="T15" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="U15" s="14">
+        <v>3</v>
+      </c>
+      <c r="V15" s="14" t="s">
+        <v>107</v>
+      </c>
       <c r="W15" s="17"/>
     </row>
-    <row r="16" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="10">
         <v>7</v>
       </c>
       <c r="B16" s="23"/>
-      <c r="C16" s="15" t="s">
-        <v>49</v>
+      <c r="C16" s="35" t="s">
+        <v>48</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E16" s="13"/>
-      <c r="F16" s="11"/>
+      <c r="F16" s="32"/>
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
-      <c r="I16" s="11"/>
+      <c r="I16" s="31"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13"/>
-      <c r="L16" s="11"/>
+      <c r="L16" s="31"/>
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
-      <c r="O16" s="11"/>
+      <c r="O16" s="31"/>
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
-      <c r="R16" s="11"/>
+      <c r="R16" s="31"/>
       <c r="S16" s="13"/>
       <c r="T16" s="13"/>
       <c r="U16" s="13"/>
       <c r="V16" s="13"/>
       <c r="W16" s="16"/>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A17" s="10">
+    <row r="17" spans="1:23" s="41" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="36">
         <v>8</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="12"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="12"/>
-      <c r="P17" s="14"/>
-      <c r="Q17" s="14"/>
-      <c r="R17" s="12"/>
-      <c r="S17" s="14"/>
-      <c r="T17" s="14"/>
-      <c r="U17" s="14"/>
-      <c r="V17" s="14"/>
-      <c r="W17" s="17"/>
+      <c r="B17" s="37">
+        <f>B15+1</f>
+        <v>45808</v>
+      </c>
+      <c r="C17" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="39">
+        <v>2</v>
+      </c>
+      <c r="F17" s="40" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/ransom-note/","Ransom Note")</f>
+        <v>Ransom Note</v>
+      </c>
+      <c r="G17" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="I17" s="40" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/find-the-difference/description/","FindDifference")</f>
+        <v>FindDifference</v>
+      </c>
+      <c r="J17" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="K17" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="L17" s="40" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/first-unique-character-in-a-string/","First Unique Character in a String")</f>
+        <v>First Unique Character in a String</v>
+      </c>
+      <c r="M17" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="N17" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="O17" s="40" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/word-pattern/","Word Pattern")</f>
+        <v>Word Pattern</v>
+      </c>
+      <c r="P17" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q17" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="R17" s="40" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/isomorphic-strings/","Isomorphic Strings")</f>
+        <v>Isomorphic Strings</v>
+      </c>
+      <c r="S17" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="T17" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="U17" s="39">
+        <v>2</v>
+      </c>
+      <c r="V17" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="W17" s="43">
+        <v>2916474</v>
+      </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="10">
         <v>9</v>
       </c>
-      <c r="B18" s="23"/>
+      <c r="B18" s="23">
+        <f>B17</f>
+        <v>45808</v>
+      </c>
       <c r="C18" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="13"/>
+        <v>50</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>111</v>
+      </c>
       <c r="E18" s="13"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="13"/>
-      <c r="R18" s="11"/>
-      <c r="S18" s="13"/>
-      <c r="T18" s="13"/>
-      <c r="U18" s="13"/>
-      <c r="V18" s="13"/>
-      <c r="W18" s="16"/>
+      <c r="F18" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/is-subsequence/","is-Subsequence")</f>
+        <v>is-Subsequence</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I18" s="40" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/valid-sudoku/description/","isValidSudoku")</f>
+        <v>isValidSudoku</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="L18" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/","Top K Frequent Elements")</f>
+        <v>Top K Frequent Elements</v>
+      </c>
+      <c r="M18" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N18" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="O18" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/longest-consecutive-sequence/","Longest Consecutive Sequence")</f>
+        <v>Longest Consecutive Sequence</v>
+      </c>
+      <c r="P18" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q18" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="R18" s="40" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/","LetterCombinationsNokia")</f>
+        <v>LetterCombinationsNokia</v>
+      </c>
+      <c r="S18" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="T18" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="U18" s="13">
+        <v>3</v>
+      </c>
+      <c r="V18" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="W18" s="42">
+        <v>2688647</v>
+      </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="10">
@@ -1932,7 +2114,7 @@
       </c>
       <c r="B19" s="23"/>
       <c r="C19" s="15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
@@ -1955,31 +2137,56 @@
       <c r="V19" s="14"/>
       <c r="W19" s="17"/>
     </row>
-    <row r="20" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="10">
         <v>11</v>
       </c>
       <c r="B20" s="23"/>
-      <c r="C20" s="30" t="s">
-        <v>53</v>
+      <c r="C20" s="33" t="s">
+        <v>52</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
-      <c r="F20" s="11"/>
+      <c r="F20" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/reverse-linked-list/","Reverse Linked List")</f>
+        <v>Reverse Linked List</v>
+      </c>
       <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="11"/>
+      <c r="H20" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I20" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/linked-list-cycle/","Linked List Cycle")</f>
+        <v>Linked List Cycle</v>
+      </c>
       <c r="J20" s="13"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="11"/>
+      <c r="K20" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L20" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/middle-of-the-linked-list/","Middle of the Linked List")</f>
+        <v>Middle of the Linked List</v>
+      </c>
       <c r="M20" s="13"/>
-      <c r="N20" s="13"/>
-      <c r="O20" s="11"/>
+      <c r="N20" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O20" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/intersection-of-two-linked-lists/","Intersection of Two Linked Lists")</f>
+        <v>Intersection of Two Linked Lists</v>
+      </c>
       <c r="P20" s="13"/>
-      <c r="Q20" s="13"/>
-      <c r="R20" s="11"/>
+      <c r="Q20" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="R20" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/linked-list-cycle-ii/","Linked List Cycle II")</f>
+        <v>Linked List Cycle II</v>
+      </c>
       <c r="S20" s="13"/>
-      <c r="T20" s="13"/>
+      <c r="T20" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="U20" s="13"/>
       <c r="V20" s="13"/>
       <c r="W20" s="16"/>
@@ -1990,7 +2197,7 @@
       </c>
       <c r="B21" s="23"/>
       <c r="C21" s="15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
@@ -2019,7 +2226,7 @@
       </c>
       <c r="B22" s="23"/>
       <c r="C22" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
@@ -2048,7 +2255,7 @@
       </c>
       <c r="B23" s="23"/>
       <c r="C23" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D23" s="14"/>
       <c r="E23" s="14"/>
@@ -2071,13 +2278,13 @@
       <c r="V23" s="14"/>
       <c r="W23" s="17"/>
     </row>
-    <row r="24" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="10">
         <v>15</v>
       </c>
       <c r="B24" s="23"/>
-      <c r="C24" s="15" t="s">
-        <v>57</v>
+      <c r="C24" s="35" t="s">
+        <v>56</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
@@ -2100,13 +2307,13 @@
       <c r="V24" s="13"/>
       <c r="W24" s="16"/>
     </row>
-    <row r="25" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="10">
         <v>16</v>
       </c>
       <c r="B25" s="23"/>
-      <c r="C25" s="15" t="s">
-        <v>30</v>
+      <c r="C25" s="35" t="s">
+        <v>29</v>
       </c>
       <c r="D25" s="14"/>
       <c r="E25" s="14"/>
@@ -2135,7 +2342,7 @@
       </c>
       <c r="B26" s="23"/>
       <c r="C26" s="15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
@@ -2158,13 +2365,13 @@
       <c r="V26" s="13"/>
       <c r="W26" s="16"/>
     </row>
-    <row r="27" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="10">
         <v>18</v>
       </c>
       <c r="B27" s="23"/>
-      <c r="C27" s="15" t="s">
-        <v>59</v>
+      <c r="C27" s="35" t="s">
+        <v>58</v>
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
@@ -2193,7 +2400,7 @@
       </c>
       <c r="B28" s="23"/>
       <c r="C28" s="15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
@@ -2222,7 +2429,7 @@
       </c>
       <c r="B29" s="23"/>
       <c r="C29" s="15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
@@ -2251,7 +2458,7 @@
       </c>
       <c r="B30" s="23"/>
       <c r="C30" s="15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
@@ -2280,7 +2487,7 @@
       </c>
       <c r="B31" s="23"/>
       <c r="C31" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D31" s="14"/>
       <c r="E31" s="14"/>
@@ -2309,7 +2516,7 @@
       </c>
       <c r="B32" s="23"/>
       <c r="C32" s="15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
@@ -2332,13 +2539,13 @@
       <c r="V32" s="13"/>
       <c r="W32" s="16"/>
     </row>
-    <row r="33" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="10">
         <v>24</v>
       </c>
       <c r="B33" s="23"/>
-      <c r="C33" s="15" t="s">
-        <v>65</v>
+      <c r="C33" s="35" t="s">
+        <v>64</v>
       </c>
       <c r="D33" s="14"/>
       <c r="E33" s="14"/>
@@ -2367,7 +2574,7 @@
       </c>
       <c r="B34" s="23"/>
       <c r="C34" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
@@ -2396,7 +2603,7 @@
       </c>
       <c r="B35" s="23"/>
       <c r="C35" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D35" s="14"/>
       <c r="E35" s="14"/>
@@ -2425,7 +2632,7 @@
       </c>
       <c r="B36" s="23"/>
       <c r="C36" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
@@ -2454,7 +2661,7 @@
       </c>
       <c r="B37" s="23"/>
       <c r="C37" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D37" s="14"/>
       <c r="E37" s="14"/>
@@ -2483,7 +2690,7 @@
       </c>
       <c r="B38" s="23"/>
       <c r="C38" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
@@ -2512,7 +2719,7 @@
       </c>
       <c r="B39" s="23"/>
       <c r="C39" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D39" s="14"/>
       <c r="E39" s="14"/>
@@ -2540,8 +2747,8 @@
         <v>31</v>
       </c>
       <c r="B40" s="23"/>
-      <c r="C40" s="15" t="s">
-        <v>73</v>
+      <c r="C40" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
@@ -2569,8 +2776,8 @@
         <v>32</v>
       </c>
       <c r="B41" s="23"/>
-      <c r="C41" s="15" t="s">
-        <v>74</v>
+      <c r="C41" s="35" t="s">
+        <v>73</v>
       </c>
       <c r="D41" s="14"/>
       <c r="E41" s="14"/>
@@ -2598,8 +2805,8 @@
         <v>33</v>
       </c>
       <c r="B42" s="23"/>
-      <c r="C42" s="15" t="s">
-        <v>75</v>
+      <c r="C42" s="35" t="s">
+        <v>74</v>
       </c>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
@@ -2627,8 +2834,8 @@
         <v>34</v>
       </c>
       <c r="B43" s="23"/>
-      <c r="C43" s="15" t="s">
-        <v>76</v>
+      <c r="C43" s="35" t="s">
+        <v>75</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
@@ -2656,8 +2863,8 @@
         <v>35</v>
       </c>
       <c r="B44" s="23"/>
-      <c r="C44" s="15" t="s">
-        <v>77</v>
+      <c r="C44" s="35" t="s">
+        <v>76</v>
       </c>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
@@ -2680,13 +2887,13 @@
       <c r="V44" s="13"/>
       <c r="W44" s="16"/>
     </row>
-    <row r="45" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A45" s="10">
         <v>36</v>
       </c>
       <c r="B45" s="23"/>
-      <c r="C45" s="15" t="s">
-        <v>78</v>
+      <c r="C45" s="35" t="s">
+        <v>77</v>
       </c>
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
@@ -2714,8 +2921,8 @@
         <v>37</v>
       </c>
       <c r="B46" s="23"/>
-      <c r="C46" s="15" t="s">
-        <v>79</v>
+      <c r="C46" s="35" t="s">
+        <v>78</v>
       </c>
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
@@ -2743,8 +2950,8 @@
         <v>38</v>
       </c>
       <c r="B47" s="23"/>
-      <c r="C47" s="15" t="s">
-        <v>80</v>
+      <c r="C47" s="35" t="s">
+        <v>79</v>
       </c>
       <c r="D47" s="14"/>
       <c r="E47" s="14"/>
@@ -2772,8 +2979,8 @@
         <v>39</v>
       </c>
       <c r="B48" s="23"/>
-      <c r="C48" s="15" t="s">
-        <v>81</v>
+      <c r="C48" s="35" t="s">
+        <v>80</v>
       </c>
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
@@ -2796,13 +3003,13 @@
       <c r="V48" s="13"/>
       <c r="W48" s="16"/>
     </row>
-    <row r="49" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A49" s="10">
         <v>40</v>
       </c>
       <c r="B49" s="23"/>
-      <c r="C49" s="15" t="s">
-        <v>82</v>
+      <c r="C49" s="35" t="s">
+        <v>81</v>
       </c>
       <c r="D49" s="14"/>
       <c r="E49" s="14"/>
@@ -2830,8 +3037,8 @@
         <v>41</v>
       </c>
       <c r="B50" s="23"/>
-      <c r="C50" s="15" t="s">
-        <v>83</v>
+      <c r="C50" s="35" t="s">
+        <v>82</v>
       </c>
       <c r="D50" s="13"/>
       <c r="E50" s="13"/>
@@ -2859,8 +3066,8 @@
         <v>42</v>
       </c>
       <c r="B51" s="23"/>
-      <c r="C51" s="15" t="s">
-        <v>84</v>
+      <c r="C51" s="35" t="s">
+        <v>83</v>
       </c>
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
@@ -2888,8 +3095,8 @@
         <v>43</v>
       </c>
       <c r="B52" s="23"/>
-      <c r="C52" s="15" t="s">
-        <v>85</v>
+      <c r="C52" s="35" t="s">
+        <v>84</v>
       </c>
       <c r="D52" s="13"/>
       <c r="E52" s="13"/>
@@ -2917,8 +3124,8 @@
         <v>44</v>
       </c>
       <c r="B53" s="23"/>
-      <c r="C53" s="15" t="s">
-        <v>86</v>
+      <c r="C53" s="35" t="s">
+        <v>85</v>
       </c>
       <c r="D53" s="14"/>
       <c r="E53" s="14"/>
@@ -2946,8 +3153,8 @@
         <v>45</v>
       </c>
       <c r="B54" s="23"/>
-      <c r="C54" s="15" t="s">
-        <v>87</v>
+      <c r="C54" s="35" t="s">
+        <v>86</v>
       </c>
       <c r="D54" s="13"/>
       <c r="E54" s="13"/>
@@ -2975,8 +3182,8 @@
         <v>46</v>
       </c>
       <c r="B55" s="23"/>
-      <c r="C55" s="15" t="s">
-        <v>88</v>
+      <c r="C55" s="35" t="s">
+        <v>87</v>
       </c>
       <c r="D55" s="14"/>
       <c r="E55" s="14"/>
@@ -3004,8 +3211,8 @@
         <v>47</v>
       </c>
       <c r="B56" s="23"/>
-      <c r="C56" s="15" t="s">
-        <v>89</v>
+      <c r="C56" s="35" t="s">
+        <v>88</v>
       </c>
       <c r="D56" s="13"/>
       <c r="E56" s="13"/>
@@ -3033,8 +3240,8 @@
         <v>48</v>
       </c>
       <c r="B57" s="23"/>
-      <c r="C57" s="15" t="s">
-        <v>90</v>
+      <c r="C57" s="35" t="s">
+        <v>89</v>
       </c>
       <c r="D57" s="14"/>
       <c r="E57" s="14"/>
@@ -3062,8 +3269,8 @@
         <v>49</v>
       </c>
       <c r="B58" s="23"/>
-      <c r="C58" s="15" t="s">
-        <v>91</v>
+      <c r="C58" s="35" t="s">
+        <v>90</v>
       </c>
       <c r="D58" s="13"/>
       <c r="E58" s="13"/>
@@ -3091,8 +3298,8 @@
         <v>50</v>
       </c>
       <c r="B59" s="23"/>
-      <c r="C59" s="15" t="s">
-        <v>92</v>
+      <c r="C59" s="35" t="s">
+        <v>91</v>
       </c>
       <c r="D59" s="14"/>
       <c r="E59" s="14"/>
@@ -3115,13 +3322,13 @@
       <c r="V59" s="14"/>
       <c r="W59" s="17"/>
     </row>
-    <row r="60" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A60" s="10">
         <v>51</v>
       </c>
       <c r="B60" s="23"/>
-      <c r="C60" s="15" t="s">
-        <v>93</v>
+      <c r="C60" s="35" t="s">
+        <v>92</v>
       </c>
       <c r="D60" s="13"/>
       <c r="E60" s="13"/>
@@ -3149,8 +3356,8 @@
         <v>52</v>
       </c>
       <c r="B61" s="23"/>
-      <c r="C61" s="15" t="s">
-        <v>94</v>
+      <c r="C61" s="35" t="s">
+        <v>93</v>
       </c>
       <c r="D61" s="14"/>
       <c r="E61" s="14"/>
@@ -3178,8 +3385,8 @@
         <v>53</v>
       </c>
       <c r="B62" s="23"/>
-      <c r="C62" s="15" t="s">
-        <v>95</v>
+      <c r="C62" s="35" t="s">
+        <v>94</v>
       </c>
       <c r="D62" s="13"/>
       <c r="E62" s="13"/>
@@ -3207,8 +3414,8 @@
         <v>54</v>
       </c>
       <c r="B63" s="23"/>
-      <c r="C63" s="15" t="s">
-        <v>96</v>
+      <c r="C63" s="35" t="s">
+        <v>95</v>
       </c>
       <c r="D63" s="14"/>
       <c r="E63" s="14"/>
@@ -3231,13 +3438,13 @@
       <c r="V63" s="14"/>
       <c r="W63" s="17"/>
     </row>
-    <row r="64" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A64" s="10">
         <v>55</v>
       </c>
       <c r="B64" s="23"/>
       <c r="C64" s="15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D64" s="13"/>
       <c r="E64" s="13"/>
@@ -3260,13 +3467,13 @@
       <c r="V64" s="13"/>
       <c r="W64" s="16"/>
     </row>
-    <row r="65" spans="1:23" ht="29" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A65" s="10">
         <v>56</v>
       </c>
       <c r="B65" s="23"/>
       <c r="C65" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D65" s="14"/>
       <c r="E65" s="14"/>
@@ -3295,7 +3502,7 @@
       </c>
       <c r="B66" s="23"/>
       <c r="C66" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D66" s="13"/>
       <c r="E66" s="13"/>
@@ -3324,7 +3531,7 @@
       </c>
       <c r="B67" s="23"/>
       <c r="C67" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D67" s="14"/>
       <c r="E67" s="14"/>
@@ -3353,7 +3560,7 @@
       </c>
       <c r="B68" s="23"/>
       <c r="C68" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D68" s="13"/>
       <c r="E68" s="13"/>
@@ -3382,7 +3589,7 @@
       </c>
       <c r="B69" s="23"/>
       <c r="C69" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D69" s="14"/>
       <c r="E69" s="14"/>
@@ -3407,48 +3614,48 @@
     </row>
     <row r="71" spans="1:23" ht="16" x14ac:dyDescent="0.4">
       <c r="A71" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
+        <v>31</v>
+      </c>
+      <c r="B72" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="B72" s="18" t="s">
+      <c r="C72" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C72" s="19" t="s">
+      <c r="D72" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="D72" s="20" t="s">
+      <c r="E72" s="21" t="s">
         <v>35</v>
-      </c>
-      <c r="E72" s="21" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="73" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
+        <v>36</v>
+      </c>
+      <c r="B73" s="27" t="s">
         <v>37</v>
-      </c>
-      <c r="B73" s="27" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="74" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
+        <v>38</v>
+      </c>
+      <c r="B74" s="27" t="s">
         <v>39</v>
-      </c>
-      <c r="B74" s="27" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="75" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B75" s="27" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Linked list and recursion practice files, implement helper utility, and update hashing notebook with improved debugging output
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1597EC-5F82-455F-8EC1-64941F817800}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88567E74-E88E-42C2-878F-A3CB84A4906D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
+    <workbookView xWindow="22932" yWindow="-1416" windowWidth="23256" windowHeight="12456" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="115">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -403,6 +403,9 @@
   </si>
   <si>
     <t>~35 Lakhs</t>
+  </si>
+  <si>
+    <t>4E-1M</t>
   </si>
 </sst>
 </file>
@@ -545,7 +548,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -630,6 +633,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -659,7 +668,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -745,29 +754,16 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1352,7 +1348,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="526" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="437" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1384,19 +1380,19 @@
     <col min="5" max="5" width="14.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.26953125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.36328125" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="21.81640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.26953125" customWidth="1"/>
+    <col min="11" max="11" width="9.26953125" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="23.54296875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.36328125" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="23.36328125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.6328125" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="21.26953125" customWidth="1"/>
     <col min="19" max="19" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.6328125" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="14.90625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="12.90625" bestFit="1" customWidth="1"/>
@@ -1432,14 +1428,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.11666666666666667</v>
+        <v>0.13333333333333333</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1448,21 +1444,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.7142857142857144</v>
+        <v>2.625</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="17" x14ac:dyDescent="0.4">
@@ -1546,7 +1542,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="23">
-        <v>45803</v>
+        <v>46168</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>42</v>
@@ -1613,7 +1609,7 @@
       <c r="V10" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W10" s="44" t="s">
+      <c r="W10" s="38" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1622,7 +1618,7 @@
         <v>2</v>
       </c>
       <c r="B11" s="23">
-        <v>45804</v>
+        <v>46169</v>
       </c>
       <c r="C11" s="15" t="s">
         <v>43</v>
@@ -1697,7 +1693,7 @@
       </c>
       <c r="B12" s="23">
         <f>B11+1</f>
-        <v>45805</v>
+        <v>46170</v>
       </c>
       <c r="C12" s="15" t="s">
         <v>44</v>
@@ -1781,7 +1777,7 @@
       </c>
       <c r="B14" s="23">
         <f>B12+1</f>
-        <v>45806</v>
+        <v>46171</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>46</v>
@@ -1856,7 +1852,7 @@
       </c>
       <c r="B15" s="23">
         <f>B14+1</f>
-        <v>45807</v>
+        <v>46172</v>
       </c>
       <c r="C15" s="15" t="s">
         <v>47</v>
@@ -1937,99 +1933,99 @@
         <v>110</v>
       </c>
       <c r="E16" s="13"/>
-      <c r="F16" s="32"/>
+      <c r="F16" s="11"/>
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
-      <c r="I16" s="31"/>
+      <c r="I16" s="11"/>
       <c r="J16" s="13"/>
       <c r="K16" s="13"/>
-      <c r="L16" s="31"/>
+      <c r="L16" s="11"/>
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
-      <c r="O16" s="31"/>
+      <c r="O16" s="11"/>
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
-      <c r="R16" s="31"/>
+      <c r="R16" s="11"/>
       <c r="S16" s="13"/>
       <c r="T16" s="13"/>
       <c r="U16" s="13"/>
       <c r="V16" s="13"/>
       <c r="W16" s="16"/>
     </row>
-    <row r="17" spans="1:23" s="41" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="36">
+    <row r="17" spans="1:23" s="36" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="10">
         <v>8</v>
       </c>
-      <c r="B17" s="37">
+      <c r="B17" s="23">
         <f>B15+1</f>
-        <v>45808</v>
-      </c>
-      <c r="C17" s="38" t="s">
+        <v>46173</v>
+      </c>
+      <c r="C17" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="39" t="s">
+      <c r="D17" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="39">
+      <c r="E17" s="14">
         <v>2</v>
       </c>
-      <c r="F17" s="40" t="str">
+      <c r="F17" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/ransom-note/","Ransom Note")</f>
         <v>Ransom Note</v>
       </c>
-      <c r="G17" s="39" t="s">
+      <c r="G17" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="H17" s="39" t="s">
+      <c r="H17" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="I17" s="40" t="str">
+      <c r="I17" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/find-the-difference/description/","FindDifference")</f>
         <v>FindDifference</v>
       </c>
-      <c r="J17" s="39" t="s">
+      <c r="J17" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="K17" s="39" t="s">
+      <c r="K17" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="L17" s="40" t="str">
+      <c r="L17" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/first-unique-character-in-a-string/","First Unique Character in a String")</f>
         <v>First Unique Character in a String</v>
       </c>
-      <c r="M17" s="39" t="s">
+      <c r="M17" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="N17" s="39" t="s">
+      <c r="N17" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="O17" s="40" t="str">
+      <c r="O17" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/word-pattern/","Word Pattern")</f>
         <v>Word Pattern</v>
       </c>
-      <c r="P17" s="39" t="s">
+      <c r="P17" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="Q17" s="39" t="s">
+      <c r="Q17" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="R17" s="40" t="str">
+      <c r="R17" s="34" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/isomorphic-strings/","Isomorphic Strings")</f>
         <v>Isomorphic Strings</v>
       </c>
-      <c r="S17" s="39" t="s">
+      <c r="S17" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="T17" s="39" t="s">
+      <c r="T17" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="U17" s="39">
+      <c r="U17" s="14">
         <v>2</v>
       </c>
-      <c r="V17" s="39" t="s">
+      <c r="V17" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W17" s="43">
+      <c r="W17" s="17">
         <v>2916474</v>
       </c>
     </row>
@@ -2038,8 +2034,8 @@
         <v>9</v>
       </c>
       <c r="B18" s="23">
-        <f>B17</f>
-        <v>45808</v>
+        <f>B17+1</f>
+        <v>46174</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>50</v>
@@ -2047,55 +2043,57 @@
       <c r="D18" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E18" s="13"/>
-      <c r="F18" s="32" t="str">
+      <c r="E18" s="13">
+        <v>3</v>
+      </c>
+      <c r="F18" s="29" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/is-subsequence/","is-Subsequence")</f>
         <v>is-Subsequence</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="G18" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="13" t="s">
+      <c r="H18" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="I18" s="40" t="str">
+      <c r="I18" s="29" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/valid-sudoku/description/","isValidSudoku")</f>
         <v>isValidSudoku</v>
       </c>
-      <c r="J18" s="13" t="s">
+      <c r="J18" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="K18" s="13" t="s">
+      <c r="K18" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="L18" s="31" t="str">
+      <c r="L18" s="29" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/","Top K Frequent Elements")</f>
         <v>Top K Frequent Elements</v>
       </c>
-      <c r="M18" s="13" t="s">
+      <c r="M18" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="N18" s="13" t="s">
+      <c r="N18" s="30" t="s">
         <v>105</v>
       </c>
       <c r="O18" s="31" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/longest-consecutive-sequence/","Longest Consecutive Sequence")</f>
         <v>Longest Consecutive Sequence</v>
       </c>
-      <c r="P18" s="13" t="s">
+      <c r="P18" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="Q18" s="13" t="s">
+      <c r="Q18" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="R18" s="40" t="str">
+      <c r="R18" s="31" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/","LetterCombinationsNokia")</f>
         <v>LetterCombinationsNokia</v>
       </c>
-      <c r="S18" s="13" t="s">
+      <c r="S18" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="T18" s="13" t="s">
+      <c r="T18" s="30" t="s">
         <v>105</v>
       </c>
       <c r="U18" s="13">
@@ -2104,7 +2102,7 @@
       <c r="V18" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W18" s="42">
+      <c r="W18" s="16">
         <v>2688647</v>
       </c>
     </row>
@@ -2141,17 +2139,26 @@
       <c r="A20" s="10">
         <v>11</v>
       </c>
-      <c r="B20" s="23"/>
+      <c r="B20" s="23">
+        <f>B18+1</f>
+        <v>46175</v>
+      </c>
       <c r="C20" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
+      <c r="D20" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="13">
+        <v>4</v>
+      </c>
       <c r="F20" s="31" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/reverse-linked-list/","Reverse Linked List")</f>
         <v>Reverse Linked List</v>
       </c>
-      <c r="G20" s="13"/>
+      <c r="G20" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="H20" s="13" t="s">
         <v>106</v>
       </c>
@@ -2159,7 +2166,9 @@
         <f>HYPERLINK("https://leetcode.com/problems/linked-list-cycle/","Linked List Cycle")</f>
         <v>Linked List Cycle</v>
       </c>
-      <c r="J20" s="13"/>
+      <c r="J20" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="K20" s="13" t="s">
         <v>106</v>
       </c>
@@ -2167,7 +2176,9 @@
         <f>HYPERLINK("https://leetcode.com/problems/middle-of-the-linked-list/","Middle of the Linked List")</f>
         <v>Middle of the Linked List</v>
       </c>
-      <c r="M20" s="13"/>
+      <c r="M20" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="N20" s="13" t="s">
         <v>106</v>
       </c>
@@ -2175,7 +2186,9 @@
         <f>HYPERLINK("https://leetcode.com/problems/intersection-of-two-linked-lists/","Intersection of Two Linked Lists")</f>
         <v>Intersection of Two Linked Lists</v>
       </c>
-      <c r="P20" s="13"/>
+      <c r="P20" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="Q20" s="13" t="s">
         <v>106</v>
       </c>
@@ -2183,13 +2196,21 @@
         <f>HYPERLINK("https://leetcode.com/problems/linked-list-cycle-ii/","Linked List Cycle II")</f>
         <v>Linked List Cycle II</v>
       </c>
-      <c r="S20" s="13"/>
+      <c r="S20" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="T20" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="U20" s="13"/>
-      <c r="V20" s="13"/>
-      <c r="W20" s="16"/>
+      <c r="U20" s="13">
+        <v>2</v>
+      </c>
+      <c r="V20" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="W20" s="37">
+        <v>2518417</v>
+      </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="10">
@@ -2199,23 +2220,50 @@
       <c r="C21" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="D21" s="14"/>
+      <c r="D21" s="14" t="s">
+        <v>114</v>
+      </c>
       <c r="E21" s="14"/>
-      <c r="F21" s="12"/>
+      <c r="F21" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/","Merge Two Sorted Lists")</f>
+        <v>Merge Two Sorted Lists</v>
+      </c>
       <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="12"/>
+      <c r="H21" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="I21" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/remove-linked-list-elements/","Remove Linked List Elements")</f>
+        <v>Remove Linked List Elements</v>
+      </c>
       <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="12"/>
+      <c r="K21" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L21" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/remove-duplicates-from-sorted-list/","Remove Duplicates from Sorted List")</f>
+        <v>Remove Duplicates from Sorted List</v>
+      </c>
       <c r="M21" s="14"/>
-      <c r="N21" s="14"/>
-      <c r="O21" s="12"/>
+      <c r="N21" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="O21" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/sort-list/","Sort List")</f>
+        <v>Sort List</v>
+      </c>
       <c r="P21" s="14"/>
-      <c r="Q21" s="14"/>
-      <c r="R21" s="12"/>
+      <c r="Q21" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="R21" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/palindrome-linked-list/","Palindrome Linked List")</f>
+        <v>Palindrome Linked List</v>
+      </c>
       <c r="S21" s="14"/>
-      <c r="T21" s="14"/>
+      <c r="T21" s="14" t="s">
+        <v>106</v>
+      </c>
       <c r="U21" s="14"/>
       <c r="V21" s="14"/>
       <c r="W21" s="17"/>
@@ -2573,7 +2621,7 @@
         <v>25</v>
       </c>
       <c r="B34" s="23"/>
-      <c r="C34" s="15" t="s">
+      <c r="C34" s="39" t="s">
         <v>65</v>
       </c>
       <c r="D34" s="13"/>
@@ -2602,7 +2650,7 @@
         <v>26</v>
       </c>
       <c r="B35" s="23"/>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="39" t="s">
         <v>66</v>
       </c>
       <c r="D35" s="14"/>

</xml_diff>

<commit_message>
Linked list Merge, sort & intersection
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88567E74-E88E-42C2-878F-A3CB84A4906D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70C99C9-D57C-42C4-BDE1-BFB14DF87A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-1416" windowWidth="23256" windowHeight="12456" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="120">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -406,18 +407,35 @@
   </si>
   <si>
     <t>4E-1M</t>
+  </si>
+  <si>
+    <t>Flatten a Multilevel Doubly Linked List</t>
+  </si>
+  <si>
+    <t>Reverse a Doubly Linked List</t>
+  </si>
+  <si>
+    <t>Delete a Node in Doubly Linked List</t>
+  </si>
+  <si>
+    <t>Insert a Node in Doubly Linked List</t>
+  </si>
+  <si>
+    <t>Find Pairs with Given Sum in DLL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="dd/mmm/yyyy"/>
+    <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -547,6 +565,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="16">
     <fill>
@@ -664,11 +689,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -765,8 +791,18 @@
     <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -1348,7 +1384,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="437" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1428,14 +1464,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.13333333333333333</v>
+        <v>0.14666666666666667</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1458,7 +1494,7 @@
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.625</v>
+        <v>2.6666666666666665</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="17" x14ac:dyDescent="0.4">
@@ -2025,7 +2061,7 @@
       <c r="V17" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W17" s="17">
+      <c r="W17" s="40">
         <v>2916474</v>
       </c>
     </row>
@@ -2102,7 +2138,7 @@
       <c r="V18" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W18" s="16">
+      <c r="W18" s="41">
         <v>2688647</v>
       </c>
     </row>
@@ -2216,7 +2252,10 @@
       <c r="A21" s="10">
         <v>12</v>
       </c>
-      <c r="B21" s="23"/>
+      <c r="B21" s="23">
+        <f>B20+1</f>
+        <v>46176</v>
+      </c>
       <c r="C21" s="15" t="s">
         <v>53</v>
       </c>
@@ -2228,7 +2267,9 @@
         <f>HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/","Merge Two Sorted Lists")</f>
         <v>Merge Two Sorted Lists</v>
       </c>
-      <c r="G21" s="14"/>
+      <c r="G21" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="H21" s="14" t="s">
         <v>106</v>
       </c>
@@ -2236,7 +2277,9 @@
         <f>HYPERLINK("https://leetcode.com/problems/remove-linked-list-elements/","Remove Linked List Elements")</f>
         <v>Remove Linked List Elements</v>
       </c>
-      <c r="J21" s="14"/>
+      <c r="J21" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="K21" s="14" t="s">
         <v>106</v>
       </c>
@@ -2244,7 +2287,9 @@
         <f>HYPERLINK("https://leetcode.com/problems/remove-duplicates-from-sorted-list/","Remove Duplicates from Sorted List")</f>
         <v>Remove Duplicates from Sorted List</v>
       </c>
-      <c r="M21" s="14"/>
+      <c r="M21" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="N21" s="14" t="s">
         <v>106</v>
       </c>
@@ -2264,9 +2309,13 @@
       <c r="T21" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="U21" s="14"/>
+      <c r="U21" s="14">
+        <v>3</v>
+      </c>
       <c r="V21" s="14"/>
-      <c r="W21" s="17"/>
+      <c r="W21" s="42">
+        <v>2308118</v>
+      </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="10">
@@ -2276,23 +2325,47 @@
       <c r="C22" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="13"/>
+      <c r="D22" s="13" t="s">
+        <v>114</v>
+      </c>
       <c r="E22" s="13"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="11"/>
+      <c r="F22" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I22" s="31" t="s">
+        <v>117</v>
+      </c>
       <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="11"/>
+      <c r="K22" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L22" s="31" t="s">
+        <v>118</v>
+      </c>
       <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="11"/>
+      <c r="N22" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O22" s="31" t="s">
+        <v>119</v>
+      </c>
       <c r="P22" s="13"/>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="11"/>
+      <c r="Q22" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="R22" s="31" t="s">
+        <v>115</v>
+      </c>
       <c r="S22" s="13"/>
-      <c r="T22" s="13"/>
+      <c r="T22" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="U22" s="13"/>
       <c r="V22" s="13"/>
       <c r="W22" s="16"/>
@@ -3788,14 +3861,14 @@
       <formula>NOT(ISERROR(SEARCH("Missed",V10)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J14:J69 M14:M69 P14:P69 S14:S69 S10:S12 P10:P12 M10:M12 J10:J12 G10:G12 G14:G69" xr:uid="{E9D55A71-CD17-44C2-A5C0-197B57D54800}">
       <formula1>"Solved,Partial,Stuck,Skipped"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K14:K69 N14:N69 Q14:Q69 T14:T69 T10:T12 Q10:Q12 N10:N12 K10:K12 H10:H12 H14:H69" xr:uid="{CAA1AB83-869C-40C8-B4BF-ABCC46363A0C}">
       <formula1>"Easy,Medium,Hard"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10:D12 D14:D69" xr:uid="{EB8389DE-9A7E-4BE0-A0CD-E46497E667CE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10:D11" xr:uid="{EB8389DE-9A7E-4BE0-A0CD-E46497E667CE}">
       <formula1>"2E-2M-1H,1E-3M-1H,3E-2M,2M-3H,1E-2M-2H,All Easy,All Medium,Mock"</formula1>
     </dataValidation>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U10:U12 U14:U69" xr:uid="{94F8B5A5-4188-4E83-BA45-970C2B3977DA}">
@@ -3805,7 +3878,17 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V12 V14:V69" xr:uid="{3B5CC177-382D-4CF3-B586-1836A6C5F18E}">
       <formula1>"Not Started,In Progress,Done,Missed"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D12:D69" xr:uid="{1EFF83AC-E9C6-42CF-B81B-1CB7B4CCE23A}">
+      <formula1>"2E-2M-1H,1E-3M-1H,3E-2M,4E-1M,2M-3H,1E-2M-2H,All Easy,All Medium,Mock"</formula1>
+    </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="F22" r:id="rId1" xr:uid="{0BCAA563-C84F-4E8C-885E-E6612440D2C9}"/>
+    <hyperlink ref="I22" r:id="rId2" xr:uid="{A97A7AEC-4D46-4367-8132-822DB0C992EA}"/>
+    <hyperlink ref="L22" r:id="rId3" xr:uid="{EB8A19E1-6C17-4DDC-BAA5-9A6D5F033FDB}"/>
+    <hyperlink ref="O22" r:id="rId4" xr:uid="{A61AC803-105B-4C74-9901-5C0392E05050}"/>
+    <hyperlink ref="R22" r:id="rId5" xr:uid="{CC28259A-3368-425F-ACD0-C7D3AFA79CAB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: reorganize LinkedList DSA practice notebooks and update progress tracker
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70C99C9-D57C-42C4-BDE1-BFB14DF87A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684E04F7-7C99-4A1D-9E3F-1C240B3A3814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="120">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -654,13 +654,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <fgColor theme="3" tint="0.89999084444715716"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -781,14 +781,13 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -798,6 +797,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1411,22 +1413,22 @@
   <cols>
     <col min="1" max="1" width="20.453125" customWidth="1"/>
     <col min="2" max="2" width="16.90625" style="22" customWidth="1"/>
-    <col min="3" max="3" width="42.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.36328125" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.6328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.26953125" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="31.08984375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="6.36328125" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="23.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="28" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="7.6328125" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="21.26953125" customWidth="1"/>
+    <col min="18" max="18" width="42" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="7.6328125" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="14.90625" bestFit="1" customWidth="1"/>
@@ -1464,14 +1466,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.14666666666666667</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1480,21 +1482,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.6666666666666665</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="17" x14ac:dyDescent="0.4">
@@ -1645,7 +1647,7 @@
       <c r="V10" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W10" s="38" t="s">
+      <c r="W10" s="37" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1988,7 +1990,7 @@
       <c r="V16" s="13"/>
       <c r="W16" s="16"/>
     </row>
-    <row r="17" spans="1:23" s="36" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="10">
         <v>8</v>
       </c>
@@ -2061,7 +2063,7 @@
       <c r="V17" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W17" s="40">
+      <c r="W17" s="39">
         <v>2916474</v>
       </c>
     </row>
@@ -2138,7 +2140,7 @@
       <c r="V18" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W18" s="41">
+      <c r="W18" s="40">
         <v>2688647</v>
       </c>
     </row>
@@ -2244,7 +2246,7 @@
       <c r="V20" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W20" s="37">
+      <c r="W20" s="36">
         <v>2518417</v>
       </c>
     </row>
@@ -2262,7 +2264,9 @@
       <c r="D21" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="E21" s="14"/>
+      <c r="E21" s="14">
+        <v>3</v>
+      </c>
       <c r="F21" s="32" t="str">
         <f>HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/","Merge Two Sorted Lists")</f>
         <v>Merge Two Sorted Lists</v>
@@ -2297,7 +2301,9 @@
         <f>HYPERLINK("https://leetcode.com/problems/sort-list/","Sort List")</f>
         <v>Sort List</v>
       </c>
-      <c r="P21" s="14"/>
+      <c r="P21" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="Q21" s="14" t="s">
         <v>105</v>
       </c>
@@ -2305,15 +2311,19 @@
         <f>HYPERLINK("https://leetcode.com/problems/palindrome-linked-list/","Palindrome Linked List")</f>
         <v>Palindrome Linked List</v>
       </c>
-      <c r="S21" s="14"/>
+      <c r="S21" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="T21" s="14" t="s">
         <v>106</v>
       </c>
       <c r="U21" s="14">
         <v>3</v>
       </c>
-      <c r="V21" s="14"/>
-      <c r="W21" s="42">
+      <c r="V21" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="W21" s="41">
         <v>2308118</v>
       </c>
     </row>
@@ -2321,14 +2331,19 @@
       <c r="A22" s="10">
         <v>13</v>
       </c>
-      <c r="B22" s="23"/>
+      <c r="B22" s="23">
+        <f>B21+1</f>
+        <v>46177</v>
+      </c>
       <c r="C22" s="15" t="s">
         <v>54</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E22" s="13"/>
+      <c r="E22" s="13">
+        <v>2</v>
+      </c>
       <c r="F22" s="31" t="s">
         <v>116</v>
       </c>
@@ -2341,32 +2356,42 @@
       <c r="I22" s="31" t="s">
         <v>117</v>
       </c>
-      <c r="J22" s="13"/>
+      <c r="J22" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="K22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="L22" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="M22" s="13"/>
+      <c r="M22" s="13" t="s">
+        <v>35</v>
+      </c>
       <c r="N22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="O22" s="31" t="s">
         <v>119</v>
       </c>
-      <c r="P22" s="13"/>
+      <c r="P22" s="13" t="s">
+        <v>35</v>
+      </c>
       <c r="Q22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="R22" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="S22" s="13"/>
+      <c r="S22" s="13" t="s">
+        <v>35</v>
+      </c>
       <c r="T22" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="U22" s="13"/>
+      <c r="U22" s="13">
+        <v>1</v>
+      </c>
       <c r="V22" s="13"/>
       <c r="W22" s="16"/>
     </row>
@@ -2694,7 +2719,7 @@
         <v>25</v>
       </c>
       <c r="B34" s="23"/>
-      <c r="C34" s="39" t="s">
+      <c r="C34" s="38" t="s">
         <v>65</v>
       </c>
       <c r="D34" s="13"/>
@@ -2723,7 +2748,7 @@
         <v>26</v>
       </c>
       <c r="B35" s="23"/>
-      <c r="C35" s="39" t="s">
+      <c r="C35" s="38" t="s">
         <v>66</v>
       </c>
       <c r="D35" s="14"/>
@@ -2752,7 +2777,7 @@
         <v>27</v>
       </c>
       <c r="B36" s="23"/>
-      <c r="C36" s="15" t="s">
+      <c r="C36" s="42" t="s">
         <v>67</v>
       </c>
       <c r="D36" s="13"/>
@@ -2781,7 +2806,7 @@
         <v>28</v>
       </c>
       <c r="B37" s="23"/>
-      <c r="C37" s="15" t="s">
+      <c r="C37" s="42" t="s">
         <v>68</v>
       </c>
       <c r="D37" s="14"/>

</xml_diff>

<commit_message>
Queue Deque and stack utility examples in notebooks
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684E04F7-7C99-4A1D-9E3F-1C240B3A3814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330004BA-C737-4397-88AA-31B8EDDCC223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -62,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="130">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -422,6 +421,36 @@
   </si>
   <si>
     <t>Find Pairs with Given Sum in DLL</t>
+  </si>
+  <si>
+    <t>Valid Parentheses</t>
+  </si>
+  <si>
+    <t>Min Stack</t>
+  </si>
+  <si>
+    <t>Baseball Game</t>
+  </si>
+  <si>
+    <t>Remove Outermost Parentheses</t>
+  </si>
+  <si>
+    <t>Make The String Great</t>
+  </si>
+  <si>
+    <t>Implement Stack using Queues</t>
+  </si>
+  <si>
+    <t>Implement Queue using Stacks</t>
+  </si>
+  <si>
+    <t>Number of Recent Calls</t>
+  </si>
+  <si>
+    <t>Moving Average from Data Stream</t>
+  </si>
+  <si>
+    <t>Sliding Window Maximum</t>
   </si>
 </sst>
 </file>
@@ -1466,14 +1495,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.16666666666666666</v>
+        <v>0.17666666666666667</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1496,7 +1525,7 @@
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.5</v>
+        <v>2.4545454545454546</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="17" x14ac:dyDescent="0.4">
@@ -2393,7 +2422,9 @@
         <v>1</v>
       </c>
       <c r="V22" s="13"/>
-      <c r="W22" s="16"/>
+      <c r="W22" s="36">
+        <v>2232799</v>
+      </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="10">
@@ -2403,24 +2434,54 @@
       <c r="C23" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="14"/>
+      <c r="D23" s="14" t="s">
+        <v>41</v>
+      </c>
       <c r="E23" s="14"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="12"/>
-      <c r="M23" s="14"/>
-      <c r="N23" s="14"/>
-      <c r="O23" s="12"/>
+      <c r="F23" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="G23" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="I23" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="K23" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L23" s="32" t="s">
+        <v>121</v>
+      </c>
+      <c r="M23" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="N23" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="O23" s="32" t="s">
+        <v>122</v>
+      </c>
       <c r="P23" s="14"/>
-      <c r="Q23" s="14"/>
-      <c r="R23" s="12"/>
+      <c r="Q23" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="R23" s="32" t="s">
+        <v>123</v>
+      </c>
       <c r="S23" s="14"/>
-      <c r="T23" s="14"/>
-      <c r="U23" s="14"/>
+      <c r="T23" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="U23" s="14">
+        <v>2</v>
+      </c>
       <c r="V23" s="14"/>
       <c r="W23" s="17"/>
     </row>
@@ -2461,23 +2522,47 @@
       <c r="C25" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="12"/>
+      <c r="D25" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="E25" s="14">
+        <v>3</v>
+      </c>
+      <c r="F25" s="32" t="s">
+        <v>125</v>
+      </c>
       <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="12"/>
+      <c r="H25" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="I25" s="32" t="s">
+        <v>126</v>
+      </c>
       <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="12"/>
+      <c r="K25" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L25" s="32" t="s">
+        <v>127</v>
+      </c>
       <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="12"/>
+      <c r="N25" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="O25" s="32" t="s">
+        <v>128</v>
+      </c>
       <c r="P25" s="14"/>
-      <c r="Q25" s="14"/>
-      <c r="R25" s="12"/>
+      <c r="Q25" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="R25" s="32" t="s">
+        <v>129</v>
+      </c>
       <c r="S25" s="14"/>
-      <c r="T25" s="14"/>
+      <c r="T25" s="14" t="s">
+        <v>105</v>
+      </c>
       <c r="U25" s="14"/>
       <c r="V25" s="14"/>
       <c r="W25" s="17"/>
@@ -3913,6 +3998,16 @@
     <hyperlink ref="L22" r:id="rId3" xr:uid="{EB8A19E1-6C17-4DDC-BAA5-9A6D5F033FDB}"/>
     <hyperlink ref="O22" r:id="rId4" xr:uid="{A61AC803-105B-4C74-9901-5C0392E05050}"/>
     <hyperlink ref="R22" r:id="rId5" xr:uid="{CC28259A-3368-425F-ACD0-C7D3AFA79CAB}"/>
+    <hyperlink ref="F23" r:id="rId6" xr:uid="{1E8812AB-2BA2-4117-9817-6A7492192CBF}"/>
+    <hyperlink ref="I23" r:id="rId7" xr:uid="{7BD90B18-C9EC-4AEF-89CB-3B64D31B752B}"/>
+    <hyperlink ref="L23" r:id="rId8" xr:uid="{4E4A8D68-3F67-4384-9E3D-1687085D2F9C}"/>
+    <hyperlink ref="O23" r:id="rId9" xr:uid="{2815FFC5-10E6-4580-AFB1-860747B0F12D}"/>
+    <hyperlink ref="R23" r:id="rId10" xr:uid="{F2B784BA-1019-4562-957F-2C1E382E0662}"/>
+    <hyperlink ref="F25" r:id="rId11" xr:uid="{92D972F4-2CF5-40EE-AF46-30EE73F286A6}"/>
+    <hyperlink ref="I25" r:id="rId12" xr:uid="{736F86C0-5873-46F5-8BC6-7F0690E09AA5}"/>
+    <hyperlink ref="L25" r:id="rId13" xr:uid="{0D989383-6FDF-47B6-80E3-2A435493AB96}"/>
+    <hyperlink ref="O25" r:id="rId14" xr:uid="{4BF18446-26BD-4AD3-BF9D-F716BD1DA8E8}"/>
+    <hyperlink ref="R25" r:id="rId15" xr:uid="{57DA53C5-D5C9-4EB7-9E5B-95529EAC0CC2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sliding window maximum and queue-based stack implementations
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330004BA-C737-4397-88AA-31B8EDDCC223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33534C5-FC50-4FE4-A307-5F4C4F28DD34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="130">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -1495,14 +1495,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.17666666666666667</v>
+        <v>0.19666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1511,21 +1511,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.4545454545454546</v>
+        <v>2.4166666666666665</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="17" x14ac:dyDescent="0.4">
@@ -2421,7 +2421,9 @@
       <c r="U22" s="13">
         <v>1</v>
       </c>
-      <c r="V22" s="13"/>
+      <c r="V22" s="13" t="s">
+        <v>107</v>
+      </c>
       <c r="W22" s="36">
         <v>2232799</v>
       </c>
@@ -2430,14 +2432,19 @@
       <c r="A23" s="10">
         <v>14</v>
       </c>
-      <c r="B23" s="23"/>
+      <c r="B23" s="23">
+        <f>B22+1</f>
+        <v>46178</v>
+      </c>
       <c r="C23" s="15" t="s">
         <v>55</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="14"/>
+      <c r="E23" s="14">
+        <v>3</v>
+      </c>
       <c r="F23" s="32" t="s">
         <v>120</v>
       </c>
@@ -2468,22 +2475,30 @@
       <c r="O23" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="P23" s="14"/>
+      <c r="P23" s="14" t="s">
+        <v>35</v>
+      </c>
       <c r="Q23" s="14" t="s">
         <v>106</v>
       </c>
       <c r="R23" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="S23" s="14"/>
+      <c r="S23" s="14" t="s">
+        <v>35</v>
+      </c>
       <c r="T23" s="14" t="s">
         <v>106</v>
       </c>
       <c r="U23" s="14">
         <v>2</v>
       </c>
-      <c r="V23" s="14"/>
-      <c r="W23" s="17"/>
+      <c r="V23" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="W23" s="41">
+        <v>2141798</v>
+      </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="10">
@@ -2518,7 +2533,10 @@
       <c r="A25" s="10">
         <v>16</v>
       </c>
-      <c r="B25" s="23"/>
+      <c r="B25" s="23">
+        <f>B23+2</f>
+        <v>46180</v>
+      </c>
       <c r="C25" s="35" t="s">
         <v>29</v>
       </c>
@@ -2531,7 +2549,9 @@
       <c r="F25" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="G25" s="14"/>
+      <c r="G25" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="H25" s="14" t="s">
         <v>106</v>
       </c>
@@ -2545,33 +2565,46 @@
       <c r="L25" s="32" t="s">
         <v>127</v>
       </c>
-      <c r="M25" s="14"/>
+      <c r="M25" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="N25" s="14" t="s">
         <v>106</v>
       </c>
       <c r="O25" s="32" t="s">
         <v>128</v>
       </c>
-      <c r="P25" s="14"/>
+      <c r="P25" s="14" t="s">
+        <v>35</v>
+      </c>
       <c r="Q25" s="14" t="s">
         <v>106</v>
       </c>
       <c r="R25" s="32" t="s">
         <v>129</v>
       </c>
-      <c r="S25" s="14"/>
+      <c r="S25" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="T25" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="U25" s="14"/>
-      <c r="V25" s="14"/>
+      <c r="U25" s="14">
+        <v>2</v>
+      </c>
+      <c r="V25" s="14" t="s">
+        <v>107</v>
+      </c>
       <c r="W25" s="17"/>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="10">
         <v>17</v>
       </c>
-      <c r="B26" s="23"/>
+      <c r="B26" s="23">
+        <f>B25+1</f>
+        <v>46181</v>
+      </c>
       <c r="C26" s="15" t="s">
         <v>57</v>
       </c>

</xml_diff>

<commit_message>
Implement recursion and backtracking modules
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33534C5-FC50-4FE4-A307-5F4C4F28DD34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE725CEA-0DD0-4240-868F-1BC6DC4A711C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="143">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -451,6 +451,45 @@
   </si>
   <si>
     <t>Sliding Window Maximum</t>
+  </si>
+  <si>
+    <t>Fibonacci Number</t>
+  </si>
+  <si>
+    <t>Power of Two</t>
+  </si>
+  <si>
+    <t>Climbing Stairs</t>
+  </si>
+  <si>
+    <t>N-th Tribonacci Number</t>
+  </si>
+  <si>
+    <t>Power of Three</t>
+  </si>
+  <si>
+    <t>Pow(x, n)</t>
+  </si>
+  <si>
+    <t>Subsets</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>K-th Symbol in Grammar</t>
+  </si>
+  <si>
+    <t>Power of Four</t>
+  </si>
+  <si>
+    <t>Find the K-th Character in String Game I</t>
+  </si>
+  <si>
+    <t>Finding 3-Digit Even Numbers</t>
+  </si>
+  <si>
+    <t>Solve subsets with recursion backtracking</t>
   </si>
 </sst>
 </file>
@@ -602,7 +641,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -687,12 +726,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.89999084444715716"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -723,7 +756,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -828,9 +861,8 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1415,7 +1447,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="514" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1437,7 +1469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E99B1C2-C176-4CCF-B3C5-DBE4B58F00CD}">
-  <dimension ref="A1:W75"/>
+  <dimension ref="A1:X75"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.453125" customWidth="1"/>
@@ -1463,9 +1495,10 @@
     <col min="21" max="21" width="14.90625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="44.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:24" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
@@ -1473,17 +1506,17 @@
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:24" ht="16" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="22" t="s">
         <v>1</v>
       </c>
@@ -1495,45 +1528,45 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.19666666666666666</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" s="22" customFormat="1" x14ac:dyDescent="0.35">
+        <v>0.22666666666666666</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="22" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.4166666666666665</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" ht="17" x14ac:dyDescent="0.4">
+        <v>2.4285714285714284</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" ht="17" x14ac:dyDescent="0.4">
       <c r="A8" s="9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:23" s="26" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:24" s="26" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="24" t="s">
         <v>8</v>
       </c>
@@ -1603,8 +1636,11 @@
       <c r="W9" s="24" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X9" s="24" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="10">
         <v>1</v>
       </c>
@@ -1679,8 +1715,9 @@
       <c r="W10" s="37" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X10" s="37"/>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="10">
         <v>2</v>
       </c>
@@ -1753,8 +1790,9 @@
         <v>107</v>
       </c>
       <c r="W11" s="17"/>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X11" s="17"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" s="10">
         <v>3</v>
       </c>
@@ -1828,8 +1866,9 @@
         <v>107</v>
       </c>
       <c r="W12" s="16"/>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X12" s="16"/>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" s="10">
         <v>4</v>
       </c>
@@ -1838,7 +1877,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14" s="10">
         <v>5</v>
       </c>
@@ -1912,8 +1951,9 @@
         <v>107</v>
       </c>
       <c r="W14" s="16"/>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X14" s="16"/>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" s="10">
         <v>6</v>
       </c>
@@ -1987,8 +2027,9 @@
         <v>107</v>
       </c>
       <c r="W15" s="17"/>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X15" s="17"/>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" s="10">
         <v>7</v>
       </c>
@@ -2018,8 +2059,9 @@
       <c r="U16" s="13"/>
       <c r="V16" s="13"/>
       <c r="W16" s="16"/>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X16" s="16"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A17" s="10">
         <v>8</v>
       </c>
@@ -2095,8 +2137,9 @@
       <c r="W17" s="39">
         <v>2916474</v>
       </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X17" s="39"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A18" s="10">
         <v>9</v>
       </c>
@@ -2172,8 +2215,9 @@
       <c r="W18" s="40">
         <v>2688647</v>
       </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X18" s="40"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A19" s="10">
         <v>10</v>
       </c>
@@ -2201,8 +2245,9 @@
       <c r="U19" s="14"/>
       <c r="V19" s="14"/>
       <c r="W19" s="17"/>
-    </row>
-    <row r="20" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="X19" s="17"/>
+    </row>
+    <row r="20" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="10">
         <v>11</v>
       </c>
@@ -2278,8 +2323,9 @@
       <c r="W20" s="36">
         <v>2518417</v>
       </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X20" s="36"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A21" s="10">
         <v>12</v>
       </c>
@@ -2355,8 +2401,9 @@
       <c r="W21" s="41">
         <v>2308118</v>
       </c>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X21" s="41"/>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A22" s="10">
         <v>13</v>
       </c>
@@ -2427,8 +2474,9 @@
       <c r="W22" s="36">
         <v>2232799</v>
       </c>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X22" s="36"/>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A23" s="10">
         <v>14</v>
       </c>
@@ -2499,8 +2547,9 @@
       <c r="W23" s="41">
         <v>2141798</v>
       </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X23" s="41"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A24" s="10">
         <v>15</v>
       </c>
@@ -2528,14 +2577,15 @@
       <c r="U24" s="13"/>
       <c r="V24" s="13"/>
       <c r="W24" s="16"/>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X24" s="16"/>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A25" s="10">
         <v>16</v>
       </c>
       <c r="B25" s="23">
-        <f>B23+2</f>
-        <v>46180</v>
+        <f>B23+1</f>
+        <v>46179</v>
       </c>
       <c r="C25" s="35" t="s">
         <v>29</v>
@@ -2558,7 +2608,9 @@
       <c r="I25" s="32" t="s">
         <v>126</v>
       </c>
-      <c r="J25" s="14"/>
+      <c r="J25" s="14" t="s">
+        <v>35</v>
+      </c>
       <c r="K25" s="14" t="s">
         <v>106</v>
       </c>
@@ -2596,79 +2648,161 @@
         <v>107</v>
       </c>
       <c r="W25" s="17"/>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X25" s="17"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A26" s="10">
         <v>17</v>
       </c>
       <c r="B26" s="23">
         <f>B25+1</f>
-        <v>46181</v>
+        <v>46180</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="13"/>
-      <c r="K26" s="13"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="13"/>
-      <c r="N26" s="13"/>
-      <c r="O26" s="11"/>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="11"/>
-      <c r="S26" s="13"/>
-      <c r="T26" s="13"/>
-      <c r="U26" s="13"/>
-      <c r="V26" s="13"/>
-      <c r="W26" s="16"/>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="D26" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E26" s="13">
+        <v>2</v>
+      </c>
+      <c r="F26" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I26" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K26" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L26" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="M26" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N26" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O26" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="P26" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q26" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="R26" s="28" t="s">
+        <v>134</v>
+      </c>
+      <c r="S26" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="T26" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="U26" s="13">
+        <v>3</v>
+      </c>
+      <c r="V26" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="W26" s="36">
+        <v>1974899</v>
+      </c>
+      <c r="X26" s="16"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A27" s="10">
         <v>18</v>
       </c>
-      <c r="B27" s="23"/>
+      <c r="B27" s="23">
+        <f>B26+1</f>
+        <v>46181</v>
+      </c>
       <c r="C27" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="D27" s="14"/>
+      <c r="D27" s="14" t="s">
+        <v>104</v>
+      </c>
       <c r="E27" s="14"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="12"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="12"/>
+      <c r="F27" s="42" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="I27" s="42" t="s">
+        <v>140</v>
+      </c>
+      <c r="J27" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K27" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L27" s="42" t="s">
+        <v>138</v>
+      </c>
       <c r="M27" s="14"/>
-      <c r="N27" s="14"/>
-      <c r="O27" s="12"/>
-      <c r="P27" s="14"/>
-      <c r="Q27" s="14"/>
-      <c r="R27" s="12"/>
+      <c r="N27" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="O27" s="42" t="s">
+        <v>141</v>
+      </c>
+      <c r="P27" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q27" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="R27" s="43" t="s">
+        <v>135</v>
+      </c>
       <c r="S27" s="14"/>
-      <c r="T27" s="14"/>
-      <c r="U27" s="14"/>
-      <c r="V27" s="14"/>
+      <c r="T27" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="U27" s="14">
+        <v>2</v>
+      </c>
+      <c r="V27" s="14" t="s">
+        <v>107</v>
+      </c>
       <c r="W27" s="17"/>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A28" s="10">
         <v>19</v>
       </c>
-      <c r="B28" s="23"/>
+      <c r="B28" s="23">
+        <f>B27+1</f>
+        <v>46182</v>
+      </c>
       <c r="C28" s="15" t="s">
         <v>59</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
-      <c r="F28" s="11"/>
+      <c r="F28" s="42" t="s">
+        <v>136</v>
+      </c>
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
       <c r="I28" s="11"/>
@@ -2686,8 +2820,11 @@
       <c r="U28" s="13"/>
       <c r="V28" s="13"/>
       <c r="W28" s="16"/>
-    </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X28" s="17" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A29" s="10">
         <v>20</v>
       </c>
@@ -2715,8 +2852,9 @@
       <c r="U29" s="14"/>
       <c r="V29" s="14"/>
       <c r="W29" s="17"/>
-    </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X29" s="17"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A30" s="10">
         <v>21</v>
       </c>
@@ -2744,8 +2882,9 @@
       <c r="U30" s="13"/>
       <c r="V30" s="13"/>
       <c r="W30" s="16"/>
-    </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X30" s="16"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A31" s="10">
         <v>22</v>
       </c>
@@ -2773,8 +2912,9 @@
       <c r="U31" s="14"/>
       <c r="V31" s="14"/>
       <c r="W31" s="17"/>
-    </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X31" s="17"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A32" s="10">
         <v>23</v>
       </c>
@@ -2802,8 +2942,9 @@
       <c r="U32" s="13"/>
       <c r="V32" s="13"/>
       <c r="W32" s="16"/>
-    </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X32" s="16"/>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A33" s="10">
         <v>24</v>
       </c>
@@ -2831,8 +2972,9 @@
       <c r="U33" s="14"/>
       <c r="V33" s="14"/>
       <c r="W33" s="17"/>
-    </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X33" s="17"/>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A34" s="10">
         <v>25</v>
       </c>
@@ -2860,8 +3002,9 @@
       <c r="U34" s="13"/>
       <c r="V34" s="13"/>
       <c r="W34" s="16"/>
-    </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X34" s="16"/>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A35" s="10">
         <v>26</v>
       </c>
@@ -2889,13 +3032,14 @@
       <c r="U35" s="14"/>
       <c r="V35" s="14"/>
       <c r="W35" s="17"/>
-    </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X35" s="17"/>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A36" s="10">
         <v>27</v>
       </c>
       <c r="B36" s="23"/>
-      <c r="C36" s="42" t="s">
+      <c r="C36" s="38" t="s">
         <v>67</v>
       </c>
       <c r="D36" s="13"/>
@@ -2918,13 +3062,14 @@
       <c r="U36" s="13"/>
       <c r="V36" s="13"/>
       <c r="W36" s="16"/>
-    </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X36" s="16"/>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A37" s="10">
         <v>28</v>
       </c>
       <c r="B37" s="23"/>
-      <c r="C37" s="42" t="s">
+      <c r="C37" s="38" t="s">
         <v>68</v>
       </c>
       <c r="D37" s="14"/>
@@ -2947,8 +3092,9 @@
       <c r="U37" s="14"/>
       <c r="V37" s="14"/>
       <c r="W37" s="17"/>
-    </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X37" s="17"/>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A38" s="10">
         <v>29</v>
       </c>
@@ -2976,8 +3122,9 @@
       <c r="U38" s="13"/>
       <c r="V38" s="13"/>
       <c r="W38" s="16"/>
-    </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X38" s="16"/>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A39" s="10">
         <v>30</v>
       </c>
@@ -3005,8 +3152,9 @@
       <c r="U39" s="14"/>
       <c r="V39" s="14"/>
       <c r="W39" s="17"/>
-    </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X39" s="17"/>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A40" s="10">
         <v>31</v>
       </c>
@@ -3034,8 +3182,9 @@
       <c r="U40" s="13"/>
       <c r="V40" s="13"/>
       <c r="W40" s="16"/>
-    </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X40" s="16"/>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A41" s="10">
         <v>32</v>
       </c>
@@ -3063,8 +3212,9 @@
       <c r="U41" s="14"/>
       <c r="V41" s="14"/>
       <c r="W41" s="17"/>
-    </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X41" s="17"/>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A42" s="10">
         <v>33</v>
       </c>
@@ -3092,8 +3242,9 @@
       <c r="U42" s="13"/>
       <c r="V42" s="13"/>
       <c r="W42" s="16"/>
-    </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X42" s="16"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A43" s="10">
         <v>34</v>
       </c>
@@ -3121,8 +3272,9 @@
       <c r="U43" s="14"/>
       <c r="V43" s="14"/>
       <c r="W43" s="17"/>
-    </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X43" s="17"/>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A44" s="10">
         <v>35</v>
       </c>
@@ -3150,8 +3302,9 @@
       <c r="U44" s="13"/>
       <c r="V44" s="13"/>
       <c r="W44" s="16"/>
-    </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X44" s="16"/>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A45" s="10">
         <v>36</v>
       </c>
@@ -3179,8 +3332,9 @@
       <c r="U45" s="14"/>
       <c r="V45" s="14"/>
       <c r="W45" s="17"/>
-    </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X45" s="17"/>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A46" s="10">
         <v>37</v>
       </c>
@@ -3208,8 +3362,9 @@
       <c r="U46" s="13"/>
       <c r="V46" s="13"/>
       <c r="W46" s="16"/>
-    </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X46" s="16"/>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A47" s="10">
         <v>38</v>
       </c>
@@ -3237,8 +3392,9 @@
       <c r="U47" s="14"/>
       <c r="V47" s="14"/>
       <c r="W47" s="17"/>
-    </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X47" s="17"/>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A48" s="10">
         <v>39</v>
       </c>
@@ -3266,8 +3422,9 @@
       <c r="U48" s="13"/>
       <c r="V48" s="13"/>
       <c r="W48" s="16"/>
-    </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X48" s="16"/>
+    </row>
+    <row r="49" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A49" s="10">
         <v>40</v>
       </c>
@@ -3295,8 +3452,9 @@
       <c r="U49" s="14"/>
       <c r="V49" s="14"/>
       <c r="W49" s="17"/>
-    </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X49" s="17"/>
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A50" s="10">
         <v>41</v>
       </c>
@@ -3324,8 +3482,9 @@
       <c r="U50" s="13"/>
       <c r="V50" s="13"/>
       <c r="W50" s="16"/>
-    </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X50" s="16"/>
+    </row>
+    <row r="51" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A51" s="10">
         <v>42</v>
       </c>
@@ -3353,8 +3512,9 @@
       <c r="U51" s="14"/>
       <c r="V51" s="14"/>
       <c r="W51" s="17"/>
-    </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X51" s="17"/>
+    </row>
+    <row r="52" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A52" s="10">
         <v>43</v>
       </c>
@@ -3382,8 +3542,9 @@
       <c r="U52" s="13"/>
       <c r="V52" s="13"/>
       <c r="W52" s="16"/>
-    </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X52" s="16"/>
+    </row>
+    <row r="53" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A53" s="10">
         <v>44</v>
       </c>
@@ -3411,8 +3572,9 @@
       <c r="U53" s="14"/>
       <c r="V53" s="14"/>
       <c r="W53" s="17"/>
-    </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X53" s="17"/>
+    </row>
+    <row r="54" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A54" s="10">
         <v>45</v>
       </c>
@@ -3440,8 +3602,9 @@
       <c r="U54" s="13"/>
       <c r="V54" s="13"/>
       <c r="W54" s="16"/>
-    </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X54" s="16"/>
+    </row>
+    <row r="55" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A55" s="10">
         <v>46</v>
       </c>
@@ -3469,8 +3632,9 @@
       <c r="U55" s="14"/>
       <c r="V55" s="14"/>
       <c r="W55" s="17"/>
-    </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X55" s="17"/>
+    </row>
+    <row r="56" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A56" s="10">
         <v>47</v>
       </c>
@@ -3498,8 +3662,9 @@
       <c r="U56" s="13"/>
       <c r="V56" s="13"/>
       <c r="W56" s="16"/>
-    </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X56" s="16"/>
+    </row>
+    <row r="57" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A57" s="10">
         <v>48</v>
       </c>
@@ -3527,8 +3692,9 @@
       <c r="U57" s="14"/>
       <c r="V57" s="14"/>
       <c r="W57" s="17"/>
-    </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X57" s="17"/>
+    </row>
+    <row r="58" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A58" s="10">
         <v>49</v>
       </c>
@@ -3556,8 +3722,9 @@
       <c r="U58" s="13"/>
       <c r="V58" s="13"/>
       <c r="W58" s="16"/>
-    </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X58" s="16"/>
+    </row>
+    <row r="59" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A59" s="10">
         <v>50</v>
       </c>
@@ -3585,8 +3752,9 @@
       <c r="U59" s="14"/>
       <c r="V59" s="14"/>
       <c r="W59" s="17"/>
-    </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X59" s="17"/>
+    </row>
+    <row r="60" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A60" s="10">
         <v>51</v>
       </c>
@@ -3614,8 +3782,9 @@
       <c r="U60" s="13"/>
       <c r="V60" s="13"/>
       <c r="W60" s="16"/>
-    </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X60" s="16"/>
+    </row>
+    <row r="61" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A61" s="10">
         <v>52</v>
       </c>
@@ -3643,8 +3812,9 @@
       <c r="U61" s="14"/>
       <c r="V61" s="14"/>
       <c r="W61" s="17"/>
-    </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X61" s="17"/>
+    </row>
+    <row r="62" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A62" s="10">
         <v>53</v>
       </c>
@@ -3672,8 +3842,9 @@
       <c r="U62" s="13"/>
       <c r="V62" s="13"/>
       <c r="W62" s="16"/>
-    </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X62" s="16"/>
+    </row>
+    <row r="63" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A63" s="10">
         <v>54</v>
       </c>
@@ -3701,8 +3872,9 @@
       <c r="U63" s="14"/>
       <c r="V63" s="14"/>
       <c r="W63" s="17"/>
-    </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X63" s="17"/>
+    </row>
+    <row r="64" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A64" s="10">
         <v>55</v>
       </c>
@@ -3730,8 +3902,9 @@
       <c r="U64" s="13"/>
       <c r="V64" s="13"/>
       <c r="W64" s="16"/>
-    </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X64" s="16"/>
+    </row>
+    <row r="65" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A65" s="10">
         <v>56</v>
       </c>
@@ -3759,8 +3932,9 @@
       <c r="U65" s="14"/>
       <c r="V65" s="14"/>
       <c r="W65" s="17"/>
-    </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X65" s="17"/>
+    </row>
+    <row r="66" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A66" s="10">
         <v>57</v>
       </c>
@@ -3788,8 +3962,9 @@
       <c r="U66" s="13"/>
       <c r="V66" s="13"/>
       <c r="W66" s="16"/>
-    </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X66" s="16"/>
+    </row>
+    <row r="67" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A67" s="10">
         <v>58</v>
       </c>
@@ -3817,8 +3992,9 @@
       <c r="U67" s="14"/>
       <c r="V67" s="14"/>
       <c r="W67" s="17"/>
-    </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X67" s="17"/>
+    </row>
+    <row r="68" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A68" s="10">
         <v>59</v>
       </c>
@@ -3846,8 +4022,9 @@
       <c r="U68" s="13"/>
       <c r="V68" s="13"/>
       <c r="W68" s="16"/>
-    </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X68" s="16"/>
+    </row>
+    <row r="69" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A69" s="10">
         <v>60</v>
       </c>
@@ -3875,13 +4052,14 @@
       <c r="U69" s="14"/>
       <c r="V69" s="14"/>
       <c r="W69" s="17"/>
-    </row>
-    <row r="71" spans="1:23" ht="16" x14ac:dyDescent="0.4">
+      <c r="X69" s="17"/>
+    </row>
+    <row r="71" spans="1:24" ht="16" x14ac:dyDescent="0.4">
       <c r="A71" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>31</v>
       </c>
@@ -3898,7 +4076,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>36</v>
       </c>
@@ -3906,7 +4084,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>38</v>
       </c>
@@ -3914,7 +4092,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>40</v>
       </c>
@@ -4041,6 +4219,17 @@
     <hyperlink ref="L25" r:id="rId13" xr:uid="{0D989383-6FDF-47B6-80E3-2A435493AB96}"/>
     <hyperlink ref="O25" r:id="rId14" xr:uid="{4BF18446-26BD-4AD3-BF9D-F716BD1DA8E8}"/>
     <hyperlink ref="R25" r:id="rId15" xr:uid="{57DA53C5-D5C9-4EB7-9E5B-95529EAC0CC2}"/>
+    <hyperlink ref="F26" r:id="rId16" xr:uid="{7231A27D-A6A1-42B1-9458-181DE1FFD8FA}"/>
+    <hyperlink ref="I26" r:id="rId17" xr:uid="{6D275812-98C6-4CA2-B722-861120F220CE}"/>
+    <hyperlink ref="L26" r:id="rId18" xr:uid="{09A1B985-1419-4B48-85F1-E46BFCED3C46}"/>
+    <hyperlink ref="O26" r:id="rId19" xr:uid="{9339A91E-98A1-494E-B373-DD41DB1E5A3C}"/>
+    <hyperlink ref="R26" r:id="rId20" xr:uid="{25C05B25-63B5-402D-80F8-50D1E2B8026F}"/>
+    <hyperlink ref="F27" r:id="rId21" xr:uid="{AE15E888-4017-4A77-8D48-5A9A8C0CDE40}"/>
+    <hyperlink ref="I27" r:id="rId22" xr:uid="{04BEC848-C8D5-42E8-9970-AA9253D6E083}"/>
+    <hyperlink ref="L27" r:id="rId23" xr:uid="{DA1DFFE1-1560-4470-94BD-3036DACA2816}"/>
+    <hyperlink ref="O27" r:id="rId24" xr:uid="{F7E8A933-2121-4BB9-A33F-0519E4335416}"/>
+    <hyperlink ref="F28" r:id="rId25" xr:uid="{F853B5DB-3667-494D-8FEE-235707180B93}"/>
+    <hyperlink ref="R27" r:id="rId26" xr:uid="{48B73BF2-BC8C-4B78-8C18-305CE5D798CF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Recursion and backtracking logic across notebooks and add binary search practice file
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE725CEA-0DD0-4240-868F-1BC6DC4A711C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BEBF387-9E3A-4DE4-8322-F37C1D9166CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -38,6 +38,136 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Dushyant Singh</author>
+  </authors>
+  <commentList>
+    <comment ref="F28" authorId="0" shapeId="0" xr:uid="{02BE3E7B-74D4-446F-BD44-C1DC4F8C020F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Dushyant Singh:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://leetcode.com/problems/subsets/</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I28" authorId="0" shapeId="0" xr:uid="{BB94A636-F1ED-4887-AB03-DF2A5A891B8F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Dushyant Singh:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://www.geeksforgeeks.org/problems/subset-sums2234/1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L28" authorId="0" shapeId="0" xr:uid="{F8038BAD-7B51-4935-BA6D-DE05A8C04606}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Dushyant Singh:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://leetcode.com/problems/letter-case-permutation/</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O28" authorId="0" shapeId="0" xr:uid="{48FC9830-1272-4224-988E-29B2FB814279}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Dushyant Singh:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://leetcode.com/problems/combinations/</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R28" authorId="0" shapeId="0" xr:uid="{8FC54704-FD08-49F9-BE27-EEB516B61CFB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Dushyant Singh:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://leetcode.com/problems/combination-sum/</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
 <metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
@@ -61,7 +191,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="153">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -490,6 +620,36 @@
   </si>
   <si>
     <t>Solve subsets with recursion backtracking</t>
+  </si>
+  <si>
+    <t>Subset Sums (GfG)</t>
+  </si>
+  <si>
+    <t>Letter Case Permutation</t>
+  </si>
+  <si>
+    <t>Combinations</t>
+  </si>
+  <si>
+    <t>Combination Sum</t>
+  </si>
+  <si>
+    <t>1E-4M</t>
+  </si>
+  <si>
+    <t>Binary Search</t>
+  </si>
+  <si>
+    <t>Search Insert Position</t>
+  </si>
+  <si>
+    <t>First Bad Version</t>
+  </si>
+  <si>
+    <t>Sqrt(x)</t>
+  </si>
+  <si>
+    <t>Find First and Last Position in Sorted Array</t>
   </si>
 </sst>
 </file>
@@ -503,7 +663,7 @@
     <numFmt numFmtId="166" formatCode="dd/mmm/yyyy"/>
     <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -639,6 +799,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="15">
@@ -1447,7 +1620,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="514" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1468,7 +1641,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E99B1C2-C176-4CCF-B3C5-DBE4B58F00CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E99B1C2-C176-4CCF-B3C5-DBE4B58F00CD}">
   <dimension ref="A1:X75"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1528,14 +1701,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.22666666666666666</v>
+        <v>0.26666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1544,21 +1717,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.4285714285714284</v>
+        <v>2.3125</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="17" x14ac:dyDescent="0.4">
@@ -2737,7 +2910,9 @@
       <c r="D27" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="E27" s="14"/>
+      <c r="E27" s="14">
+        <v>3</v>
+      </c>
       <c r="F27" s="42" t="s">
         <v>139</v>
       </c>
@@ -2759,7 +2934,9 @@
       <c r="L27" s="42" t="s">
         <v>138</v>
       </c>
-      <c r="M27" s="14"/>
+      <c r="M27" s="14" t="s">
+        <v>35</v>
+      </c>
       <c r="N27" s="14" t="s">
         <v>105</v>
       </c>
@@ -2767,7 +2944,7 @@
         <v>141</v>
       </c>
       <c r="P27" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q27" s="14" t="s">
         <v>105</v>
@@ -2775,17 +2952,21 @@
       <c r="R27" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="S27" s="14"/>
+      <c r="S27" s="14" t="s">
+        <v>35</v>
+      </c>
       <c r="T27" s="14" t="s">
         <v>105</v>
       </c>
       <c r="U27" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V27" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="W27" s="17"/>
+      <c r="W27" s="41">
+        <v>1903147</v>
+      </c>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A28" s="10">
@@ -2798,27 +2979,63 @@
       <c r="C28" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="42" t="s">
+      <c r="D28" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="E28" s="13">
+        <v>2</v>
+      </c>
+      <c r="F28" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="13"/>
-      <c r="K28" s="13"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="13"/>
-      <c r="N28" s="13"/>
-      <c r="O28" s="11"/>
-      <c r="P28" s="13"/>
-      <c r="Q28" s="13"/>
-      <c r="R28" s="11"/>
-      <c r="S28" s="13"/>
-      <c r="T28" s="13"/>
-      <c r="U28" s="13"/>
-      <c r="V28" s="13"/>
+      <c r="G28" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H28" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="I28" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="J28" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="K28" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="L28" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="M28" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="N28" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="O28" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="P28" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q28" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="R28" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="S28" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="T28" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="U28" s="13">
+        <v>1</v>
+      </c>
+      <c r="V28" s="13" t="s">
+        <v>107</v>
+      </c>
       <c r="W28" s="16"/>
       <c r="X28" s="17" t="s">
         <v>142</v>
@@ -2862,25 +3079,61 @@
       <c r="C30" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="D30" s="13"/>
+      <c r="D30" s="13" t="s">
+        <v>114</v>
+      </c>
       <c r="E30" s="13"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="13"/>
-      <c r="K30" s="13"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="13"/>
-      <c r="N30" s="13"/>
-      <c r="O30" s="11"/>
-      <c r="P30" s="13"/>
-      <c r="Q30" s="13"/>
-      <c r="R30" s="11"/>
-      <c r="S30" s="13"/>
-      <c r="T30" s="13"/>
-      <c r="U30" s="13"/>
-      <c r="V30" s="13"/>
+      <c r="F30" s="28" t="s">
+        <v>148</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H30" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I30" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K30" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L30" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="M30" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N30" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O30" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="P30" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q30" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="R30" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="S30" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="T30" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="U30" s="13">
+        <v>3</v>
+      </c>
+      <c r="V30" s="13" t="s">
+        <v>107</v>
+      </c>
       <c r="W30" s="16"/>
       <c r="X30" s="16"/>
     </row>
@@ -4230,7 +4483,17 @@
     <hyperlink ref="O27" r:id="rId24" xr:uid="{F7E8A933-2121-4BB9-A33F-0519E4335416}"/>
     <hyperlink ref="F28" r:id="rId25" xr:uid="{F853B5DB-3667-494D-8FEE-235707180B93}"/>
     <hyperlink ref="R27" r:id="rId26" xr:uid="{48B73BF2-BC8C-4B78-8C18-305CE5D798CF}"/>
+    <hyperlink ref="I28" r:id="rId27" xr:uid="{44C53BE6-EDE6-40E9-AA8D-CA9F8399166C}"/>
+    <hyperlink ref="L28" r:id="rId28" xr:uid="{B1D2BE71-7F3E-4434-9A6D-9C66220C46B5}"/>
+    <hyperlink ref="O28" r:id="rId29" xr:uid="{0F422880-4AA6-446E-948D-28CC715B0680}"/>
+    <hyperlink ref="R28" r:id="rId30" xr:uid="{7803E1BF-4AEE-4CA1-B087-BB9BBB1CB12D}"/>
+    <hyperlink ref="F30" r:id="rId31" xr:uid="{0FC7EF8B-8B19-46AD-9453-30C0BB7BB9F9}"/>
+    <hyperlink ref="I30" r:id="rId32" xr:uid="{73FB2138-40AB-44C9-A98E-F9469083F92D}"/>
+    <hyperlink ref="L30" r:id="rId33" xr:uid="{6BF58775-DCDF-4832-896C-0F8482431A47}"/>
+    <hyperlink ref="O30" r:id="rId34" xr:uid="{9CB03CF7-FE30-47C8-967A-0C5340E31744}"/>
+    <hyperlink ref="R30" r:id="rId35" xr:uid="{A9148CEC-5930-483D-A2F2-C7E66E7EAE20}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId36"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sorting algorithms and binary tree traversals & BFS code
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BEBF387-9E3A-4DE4-8322-F37C1D9166CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B15AD5CB-384D-4330-82E6-B72DEE22B643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -191,7 +191,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="168">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -650,6 +650,62 @@
   </si>
   <si>
     <t>Find First and Last Position in Sorted Array</t>
+  </si>
+  <si>
+    <t>Sort Array By Parity</t>
+  </si>
+  <si>
+    <t>Height Checker</t>
+  </si>
+  <si>
+    <t>Relative Sort Array</t>
+  </si>
+  <si>
+    <t>Sort the People</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">sorted = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF569CD6"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>False</t>
+    </r>
+  </si>
+  <si>
+    <t>Binary Tree Inorder Traversal</t>
+  </si>
+  <si>
+    <t>Binary Tree Preorder Traversal</t>
+  </si>
+  <si>
+    <t>Binary Tree Postorder Traversal</t>
+  </si>
+  <si>
+    <t>N-ary Tree Preorder Traversal</t>
+  </si>
+  <si>
+    <t>N-ary Tree Postorder Traversal</t>
+  </si>
+  <si>
+    <t>Maximum Depth of Binary Tree</t>
+  </si>
+  <si>
+    <t>Diameter of Binary Tree</t>
+  </si>
+  <si>
+    <t>Balanced Binary Tree</t>
+  </si>
+  <si>
+    <t>Minimum Depth of Binary Tree</t>
+  </si>
+  <si>
+    <t>Path Sum</t>
   </si>
 </sst>
 </file>
@@ -663,7 +719,7 @@
     <numFmt numFmtId="166" formatCode="dd/mmm/yyyy"/>
     <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -813,6 +869,18 @@
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFD4D4D4"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF569CD6"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -929,7 +997,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1036,6 +1104,10 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1701,14 +1773,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.26666666666666666</v>
+        <v>0.29333333333333333</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1717,21 +1789,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.3125</v>
+        <v>2.3529411764705883</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="17" x14ac:dyDescent="0.4">
@@ -2400,7 +2472,7 @@
       </c>
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
-      <c r="F19" s="12"/>
+      <c r="F19" s="32"/>
       <c r="G19" s="14"/>
       <c r="H19" s="14"/>
       <c r="I19" s="12"/>
@@ -3075,14 +3147,19 @@
       <c r="A30" s="10">
         <v>21</v>
       </c>
-      <c r="B30" s="23"/>
+      <c r="B30" s="23">
+        <f>B28+2</f>
+        <v>46184</v>
+      </c>
       <c r="C30" s="15" t="s">
         <v>61</v>
       </c>
       <c r="D30" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E30" s="13"/>
+      <c r="E30" s="13">
+        <v>2</v>
+      </c>
       <c r="F30" s="28" t="s">
         <v>148</v>
       </c>
@@ -3134,7 +3211,9 @@
       <c r="V30" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="W30" s="16"/>
+      <c r="W30" s="36">
+        <v>1852829</v>
+      </c>
       <c r="X30" s="16"/>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.35">
@@ -3171,30 +3250,74 @@
       <c r="A32" s="10">
         <v>23</v>
       </c>
-      <c r="B32" s="23"/>
+      <c r="B32" s="23">
+        <f>B30+2</f>
+        <v>46186</v>
+      </c>
       <c r="C32" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="13"/>
-      <c r="N32" s="13"/>
-      <c r="O32" s="11"/>
-      <c r="P32" s="13"/>
-      <c r="Q32" s="13"/>
-      <c r="R32" s="11"/>
-      <c r="S32" s="13"/>
-      <c r="T32" s="13"/>
-      <c r="U32" s="13"/>
-      <c r="V32" s="13"/>
-      <c r="W32" s="16"/>
+      <c r="D32" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E32" s="13">
+        <v>3</v>
+      </c>
+      <c r="F32" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/sort-an-array/","Merge Sort Array")</f>
+        <v>Merge Sort Array</v>
+      </c>
+      <c r="G32" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H32" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I32" s="28" t="s">
+        <v>153</v>
+      </c>
+      <c r="J32" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K32" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L32" s="28" t="s">
+        <v>154</v>
+      </c>
+      <c r="M32" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N32" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O32" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="P32" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q32" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="R32" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="S32" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="T32" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="U32" s="13">
+        <v>3</v>
+      </c>
+      <c r="V32" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="W32" s="36">
+        <v>1821083</v>
+      </c>
       <c r="X32" s="16"/>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.35">
@@ -3227,7 +3350,7 @@
       <c r="W33" s="17"/>
       <c r="X33" s="17"/>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="10">
         <v>25</v>
       </c>
@@ -3257,7 +3380,7 @@
       <c r="W34" s="16"/>
       <c r="X34" s="16"/>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10">
         <v>26</v>
       </c>
@@ -3287,7 +3410,7 @@
       <c r="W35" s="17"/>
       <c r="X35" s="17"/>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="10">
         <v>27</v>
       </c>
@@ -3297,7 +3420,9 @@
       </c>
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
-      <c r="F36" s="11"/>
+      <c r="F36" s="44" t="s">
+        <v>157</v>
+      </c>
       <c r="G36" s="13"/>
       <c r="H36" s="13"/>
       <c r="I36" s="11"/>
@@ -3317,7 +3442,7 @@
       <c r="W36" s="16"/>
       <c r="X36" s="16"/>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="10">
         <v>28</v>
       </c>
@@ -3351,30 +3476,63 @@
       <c r="A38" s="10">
         <v>29</v>
       </c>
-      <c r="B38" s="23"/>
+      <c r="B38" s="23">
+        <f>B32+3</f>
+        <v>46189</v>
+      </c>
       <c r="C38" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D38" s="13"/>
+      <c r="D38" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="E38" s="13"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="11"/>
-      <c r="J38" s="13"/>
-      <c r="K38" s="13"/>
-      <c r="L38" s="11"/>
-      <c r="M38" s="13"/>
-      <c r="N38" s="13"/>
-      <c r="O38" s="11"/>
+      <c r="F38" s="31" t="s">
+        <v>159</v>
+      </c>
+      <c r="G38" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H38" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I38" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="J38" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K38" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L38" s="31" t="s">
+        <v>160</v>
+      </c>
+      <c r="M38" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N38" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O38" s="31" t="s">
+        <v>161</v>
+      </c>
       <c r="P38" s="13"/>
-      <c r="Q38" s="13"/>
-      <c r="R38" s="11"/>
+      <c r="Q38" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="R38" s="31" t="s">
+        <v>162</v>
+      </c>
       <c r="S38" s="13"/>
-      <c r="T38" s="13"/>
+      <c r="T38" s="13" t="s">
+        <v>106</v>
+      </c>
       <c r="U38" s="13"/>
       <c r="V38" s="13"/>
-      <c r="W38" s="16"/>
+      <c r="W38" s="36">
+        <v>1743188</v>
+      </c>
       <c r="X38" s="16"/>
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.35">
@@ -3385,23 +3543,45 @@
       <c r="C39" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="D39" s="14"/>
+      <c r="D39" s="14" t="s">
+        <v>41</v>
+      </c>
       <c r="E39" s="14"/>
-      <c r="F39" s="12"/>
+      <c r="F39" s="32" t="s">
+        <v>163</v>
+      </c>
       <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="12"/>
+      <c r="H39" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="I39" s="45" t="s">
+        <v>164</v>
+      </c>
       <c r="J39" s="14"/>
-      <c r="K39" s="14"/>
-      <c r="L39" s="12"/>
+      <c r="K39" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L39" s="32" t="s">
+        <v>165</v>
+      </c>
       <c r="M39" s="14"/>
-      <c r="N39" s="14"/>
-      <c r="O39" s="12"/>
+      <c r="N39" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="O39" s="32" t="s">
+        <v>166</v>
+      </c>
       <c r="P39" s="14"/>
-      <c r="Q39" s="14"/>
-      <c r="R39" s="12"/>
+      <c r="Q39" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="R39" s="32" t="s">
+        <v>167</v>
+      </c>
       <c r="S39" s="14"/>
-      <c r="T39" s="14"/>
+      <c r="T39" s="14" t="s">
+        <v>106</v>
+      </c>
       <c r="U39" s="14"/>
       <c r="V39" s="14"/>
       <c r="W39" s="17"/>
@@ -4492,8 +4672,22 @@
     <hyperlink ref="L30" r:id="rId33" xr:uid="{6BF58775-DCDF-4832-896C-0F8482431A47}"/>
     <hyperlink ref="O30" r:id="rId34" xr:uid="{9CB03CF7-FE30-47C8-967A-0C5340E31744}"/>
     <hyperlink ref="R30" r:id="rId35" xr:uid="{A9148CEC-5930-483D-A2F2-C7E66E7EAE20}"/>
+    <hyperlink ref="I32" r:id="rId36" xr:uid="{3F89DCFC-D745-44D7-BCCB-9060032738E4}"/>
+    <hyperlink ref="L32" r:id="rId37" xr:uid="{EF002432-FFD8-4BCB-ACD0-CF58435F2106}"/>
+    <hyperlink ref="O32" r:id="rId38" xr:uid="{E1381C65-281E-45C4-82A3-9450D0121EFB}"/>
+    <hyperlink ref="R32" r:id="rId39" xr:uid="{8805D0B4-2734-4FF5-BFEB-7A70B8A9C37F}"/>
+    <hyperlink ref="I38" r:id="rId40" xr:uid="{DA1BBCB8-5947-4C2E-BB8F-9BBC54572E6D}"/>
+    <hyperlink ref="F38" r:id="rId41" xr:uid="{CD3EB9E8-58BE-4E84-817C-9D403582C02B}"/>
+    <hyperlink ref="L38" r:id="rId42" xr:uid="{46B8D8A2-0727-47C8-8A24-B52E3BD7D426}"/>
+    <hyperlink ref="O38" r:id="rId43" xr:uid="{66304EBF-5D38-48DC-B7BD-2EA5601D104A}"/>
+    <hyperlink ref="R38" r:id="rId44" xr:uid="{93F22270-F70A-4B6E-A3DB-0B57FBC181FB}"/>
+    <hyperlink ref="F39" r:id="rId45" xr:uid="{92467958-BE91-477A-8CDF-CBFD920DEBD3}"/>
+    <hyperlink ref="I39" r:id="rId46" xr:uid="{2A9C14AB-C3D3-4EFF-8D17-EA65E94D7FB3}"/>
+    <hyperlink ref="L39" r:id="rId47" xr:uid="{82E6A4D0-2092-4D43-8375-59371FA319CB}"/>
+    <hyperlink ref="O39" r:id="rId48" xr:uid="{BFF0AB17-5D82-4F1B-AC16-2DF48FF962F1}"/>
+    <hyperlink ref="R39" r:id="rId49" xr:uid="{B1B0909D-1122-4439-9F88-E6434EED9786}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId36"/>
+  <legacyDrawing r:id="rId50"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactored folders, Tree traversal notebooks and remove obsolete files
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B15AD5CB-384D-4330-82E6-B72DEE22B643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B3062C1-5470-47B0-97DA-AB8283347353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -191,7 +191,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="168">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -1773,14 +1773,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.29333333333333333</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -3539,7 +3539,10 @@
       <c r="A39" s="10">
         <v>30</v>
       </c>
-      <c r="B39" s="23"/>
+      <c r="B39" s="23">
+        <f>B38+1</f>
+        <v>46190</v>
+      </c>
       <c r="C39" s="15" t="s">
         <v>70</v>
       </c>
@@ -3550,7 +3553,9 @@
       <c r="F39" s="32" t="s">
         <v>163</v>
       </c>
-      <c r="G39" s="14"/>
+      <c r="G39" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="H39" s="14" t="s">
         <v>106</v>
       </c>
@@ -3571,7 +3576,9 @@
       <c r="O39" s="32" t="s">
         <v>166</v>
       </c>
-      <c r="P39" s="14"/>
+      <c r="P39" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="Q39" s="14" t="s">
         <v>106</v>
       </c>
@@ -3584,7 +3591,9 @@
       </c>
       <c r="U39" s="14"/>
       <c r="V39" s="14"/>
-      <c r="W39" s="17"/>
+      <c r="W39" s="41">
+        <v>1700496</v>
+      </c>
       <c r="X39" s="17"/>
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.35">
@@ -3737,7 +3746,7 @@
       <c r="W44" s="16"/>
       <c r="X44" s="16"/>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="10">
         <v>36</v>
       </c>
@@ -3767,7 +3776,7 @@
       <c r="W45" s="17"/>
       <c r="X45" s="17"/>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="10">
         <v>37</v>
       </c>

</xml_diff>

<commit_message>
BFS and DFS algorithms for binary and N-ary trees practice notebooks
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B3062C1-5470-47B0-97DA-AB8283347353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FADB0A-7F9A-4842-856B-2F5FF2E54A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -52,7 +52,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Dushyant Singh:</t>
         </r>
@@ -61,7 +61,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://leetcode.com/problems/subsets/</t>
@@ -76,7 +76,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Dushyant Singh:</t>
         </r>
@@ -85,7 +85,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://www.geeksforgeeks.org/problems/subset-sums2234/1</t>
@@ -100,7 +100,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Dushyant Singh:</t>
         </r>
@@ -109,7 +109,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://leetcode.com/problems/letter-case-permutation/</t>
@@ -124,7 +124,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Dushyant Singh:</t>
         </r>
@@ -133,7 +133,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://leetcode.com/problems/combinations/</t>
@@ -148,7 +148,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Dushyant Singh:</t>
         </r>
@@ -157,7 +157,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://leetcode.com/problems/combination-sum/</t>
@@ -191,7 +191,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="183">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -706,6 +706,51 @@
   </si>
   <si>
     <t>Path Sum</t>
+  </si>
+  <si>
+    <t>Lowest Common Ancestor of a BST</t>
+  </si>
+  <si>
+    <t>Average of Levels in Binary Tree</t>
+  </si>
+  <si>
+    <t>Binary Tree Right Side View</t>
+  </si>
+  <si>
+    <t>Lowest Common Ancestor of a Binary Tree</t>
+  </si>
+  <si>
+    <t>Serialize and Deserialize BST</t>
+  </si>
+  <si>
+    <t>2E-3M</t>
+  </si>
+  <si>
+    <t>Search in a Binary Search Tree</t>
+  </si>
+  <si>
+    <t>Range Sum of BST</t>
+  </si>
+  <si>
+    <t>Closest Binary Search Tree Value</t>
+  </si>
+  <si>
+    <t>Insert into a Binary Search Tree</t>
+  </si>
+  <si>
+    <t>Delete Node in a BST</t>
+  </si>
+  <si>
+    <t>Convert Sorted Array to BST</t>
+  </si>
+  <si>
+    <t>Minimum Absolute Difference in BST</t>
+  </si>
+  <si>
+    <t>Two Sum IV - Input is a BST</t>
+  </si>
+  <si>
+    <t>Validate Binary Search Tree</t>
   </si>
 </sst>
 </file>
@@ -841,12 +886,14 @@
       <sz val="11"/>
       <color rgb="FF0563C1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -860,14 +907,14 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
@@ -882,7 +929,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -967,6 +1014,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -997,7 +1056,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1108,6 +1167,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1773,14 +1837,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.3</v>
+        <v>0.31666666666666665</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1789,21 +1853,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.3529411764705883</v>
+        <v>2.5263157894736841</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="17" x14ac:dyDescent="0.4">
@@ -3480,7 +3544,7 @@
         <f>B32+3</f>
         <v>46189</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C38" s="47" t="s">
         <v>69</v>
       </c>
       <c r="D38" s="13" t="s">
@@ -3517,19 +3581,27 @@
       <c r="O38" s="31" t="s">
         <v>161</v>
       </c>
-      <c r="P38" s="13"/>
+      <c r="P38" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="Q38" s="13" t="s">
         <v>106</v>
       </c>
       <c r="R38" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="S38" s="13"/>
+      <c r="S38" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="T38" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="U38" s="13"/>
-      <c r="V38" s="13"/>
+      <c r="U38" s="13">
+        <v>4</v>
+      </c>
+      <c r="V38" s="13" t="s">
+        <v>107</v>
+      </c>
       <c r="W38" s="36">
         <v>1743188</v>
       </c>
@@ -3543,7 +3615,7 @@
         <f>B38+1</f>
         <v>46190</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C39" s="47" t="s">
         <v>70</v>
       </c>
       <c r="D39" s="14" t="s">
@@ -3585,12 +3657,18 @@
       <c r="R39" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="S39" s="14"/>
+      <c r="S39" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="T39" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="U39" s="14"/>
-      <c r="V39" s="14"/>
+      <c r="U39" s="14">
+        <v>4</v>
+      </c>
+      <c r="V39" s="14" t="s">
+        <v>107</v>
+      </c>
       <c r="W39" s="41">
         <v>1700496</v>
       </c>
@@ -3601,29 +3679,58 @@
         <v>31</v>
       </c>
       <c r="B40" s="23"/>
-      <c r="C40" s="35" t="s">
+      <c r="C40" s="48" t="s">
         <v>72</v>
       </c>
-      <c r="D40" s="13"/>
+      <c r="D40" s="13" t="s">
+        <v>173</v>
+      </c>
       <c r="E40" s="13"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="11"/>
+      <c r="F40" s="32" t="str">
+        <f>HYPERLINK("http://leetcode.com/problems/sum-root-to-leaf-numbers/","Sum Root to Leaf")</f>
+        <v>Sum Root to Leaf</v>
+      </c>
+      <c r="G40" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H40" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I40" s="31" t="s">
+        <v>169</v>
+      </c>
       <c r="J40" s="13"/>
-      <c r="K40" s="13"/>
-      <c r="L40" s="11"/>
-      <c r="M40" s="13"/>
-      <c r="N40" s="13"/>
-      <c r="O40" s="11"/>
+      <c r="K40" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L40" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="M40" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N40" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="O40" s="31" t="s">
+        <v>171</v>
+      </c>
       <c r="P40" s="13"/>
-      <c r="Q40" s="13"/>
-      <c r="R40" s="11"/>
+      <c r="Q40" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="R40" s="31" t="s">
+        <v>172</v>
+      </c>
       <c r="S40" s="13"/>
-      <c r="T40" s="13"/>
+      <c r="T40" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="U40" s="13"/>
       <c r="V40" s="13"/>
-      <c r="W40" s="16"/>
+      <c r="W40" s="36">
+        <v>1647433</v>
+      </c>
       <c r="X40" s="16"/>
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.35">
@@ -3631,26 +3738,48 @@
         <v>32</v>
       </c>
       <c r="B41" s="23"/>
-      <c r="C41" s="35" t="s">
+      <c r="C41" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="D41" s="14"/>
+      <c r="D41" s="14" t="s">
+        <v>104</v>
+      </c>
       <c r="E41" s="14"/>
-      <c r="F41" s="12"/>
+      <c r="F41" s="32" t="s">
+        <v>174</v>
+      </c>
       <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="12"/>
+      <c r="H41" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="I41" s="32" t="s">
+        <v>175</v>
+      </c>
       <c r="J41" s="14"/>
-      <c r="K41" s="14"/>
-      <c r="L41" s="12"/>
+      <c r="K41" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L41" s="32" t="s">
+        <v>176</v>
+      </c>
       <c r="M41" s="14"/>
-      <c r="N41" s="14"/>
-      <c r="O41" s="12"/>
+      <c r="N41" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="O41" s="32" t="s">
+        <v>177</v>
+      </c>
       <c r="P41" s="14"/>
-      <c r="Q41" s="14"/>
-      <c r="R41" s="12"/>
+      <c r="Q41" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="R41" s="32" t="s">
+        <v>178</v>
+      </c>
       <c r="S41" s="14"/>
-      <c r="T41" s="14"/>
+      <c r="T41" s="14" t="s">
+        <v>105</v>
+      </c>
       <c r="U41" s="14"/>
       <c r="V41" s="14"/>
       <c r="W41" s="17"/>
@@ -3661,26 +3790,48 @@
         <v>33</v>
       </c>
       <c r="B42" s="23"/>
-      <c r="C42" s="35" t="s">
+      <c r="C42" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="D42" s="13"/>
+      <c r="D42" s="13" t="s">
+        <v>104</v>
+      </c>
       <c r="E42" s="13"/>
-      <c r="F42" s="11"/>
+      <c r="F42" s="31" t="s">
+        <v>179</v>
+      </c>
       <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="11"/>
+      <c r="H42" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I42" s="31" t="s">
+        <v>180</v>
+      </c>
       <c r="J42" s="13"/>
-      <c r="K42" s="13"/>
-      <c r="L42" s="11"/>
+      <c r="K42" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L42" s="31" t="s">
+        <v>181</v>
+      </c>
       <c r="M42" s="13"/>
-      <c r="N42" s="13"/>
-      <c r="O42" s="11"/>
+      <c r="N42" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O42" s="31" t="s">
+        <v>182</v>
+      </c>
       <c r="P42" s="13"/>
-      <c r="Q42" s="13"/>
-      <c r="R42" s="11"/>
+      <c r="Q42" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="R42" s="31" t="s">
+        <v>168</v>
+      </c>
       <c r="S42" s="13"/>
-      <c r="T42" s="13"/>
+      <c r="T42" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="U42" s="13"/>
       <c r="V42" s="13"/>
       <c r="W42" s="16"/>
@@ -3726,7 +3877,6 @@
       </c>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
-      <c r="F44" s="11"/>
       <c r="G44" s="13"/>
       <c r="H44" s="13"/>
       <c r="I44" s="11"/>
@@ -3735,7 +3885,6 @@
       <c r="L44" s="11"/>
       <c r="M44" s="13"/>
       <c r="N44" s="13"/>
-      <c r="O44" s="11"/>
       <c r="P44" s="13"/>
       <c r="Q44" s="13"/>
       <c r="R44" s="11"/>
@@ -3811,7 +3960,7 @@
         <v>38</v>
       </c>
       <c r="B47" s="23"/>
-      <c r="C47" s="35" t="s">
+      <c r="C47" s="46" t="s">
         <v>79</v>
       </c>
       <c r="D47" s="14"/>
@@ -3841,7 +3990,7 @@
         <v>39</v>
       </c>
       <c r="B48" s="23"/>
-      <c r="C48" s="35" t="s">
+      <c r="C48" s="46" t="s">
         <v>80</v>
       </c>
       <c r="D48" s="13"/>
@@ -3871,7 +4020,7 @@
         <v>40</v>
       </c>
       <c r="B49" s="23"/>
-      <c r="C49" s="35" t="s">
+      <c r="C49" s="46" t="s">
         <v>81</v>
       </c>
       <c r="D49" s="14"/>
@@ -3901,7 +4050,7 @@
         <v>41</v>
       </c>
       <c r="B50" s="23"/>
-      <c r="C50" s="35" t="s">
+      <c r="C50" s="46" t="s">
         <v>82</v>
       </c>
       <c r="D50" s="13"/>
@@ -3931,7 +4080,7 @@
         <v>42</v>
       </c>
       <c r="B51" s="23"/>
-      <c r="C51" s="35" t="s">
+      <c r="C51" s="46" t="s">
         <v>83</v>
       </c>
       <c r="D51" s="14"/>
@@ -3961,7 +4110,7 @@
         <v>43</v>
       </c>
       <c r="B52" s="23"/>
-      <c r="C52" s="35" t="s">
+      <c r="C52" s="46" t="s">
         <v>84</v>
       </c>
       <c r="D52" s="13"/>
@@ -3991,7 +4140,7 @@
         <v>44</v>
       </c>
       <c r="B53" s="23"/>
-      <c r="C53" s="35" t="s">
+      <c r="C53" s="46" t="s">
         <v>85</v>
       </c>
       <c r="D53" s="14"/>
@@ -4021,7 +4170,7 @@
         <v>45</v>
       </c>
       <c r="B54" s="23"/>
-      <c r="C54" s="35" t="s">
+      <c r="C54" s="46" t="s">
         <v>86</v>
       </c>
       <c r="D54" s="13"/>
@@ -4695,8 +4844,22 @@
     <hyperlink ref="L39" r:id="rId47" xr:uid="{82E6A4D0-2092-4D43-8375-59371FA319CB}"/>
     <hyperlink ref="O39" r:id="rId48" xr:uid="{BFF0AB17-5D82-4F1B-AC16-2DF48FF962F1}"/>
     <hyperlink ref="R39" r:id="rId49" xr:uid="{B1B0909D-1122-4439-9F88-E6434EED9786}"/>
+    <hyperlink ref="R42" r:id="rId50" xr:uid="{390735D0-260B-4FCE-8010-1BBC0F3806F5}"/>
+    <hyperlink ref="I40" r:id="rId51" xr:uid="{9616543C-4BDC-4DF6-933F-74D5C625BF36}"/>
+    <hyperlink ref="L40" r:id="rId52" xr:uid="{6AE4C4FC-0187-4F62-B77D-664FD2E68DD0}"/>
+    <hyperlink ref="O40" r:id="rId53" xr:uid="{9EECE6D1-8B47-42E8-A086-350CD43DDD65}"/>
+    <hyperlink ref="R40" r:id="rId54" xr:uid="{C3188B70-74AE-4E45-9839-E4E665756EDD}"/>
+    <hyperlink ref="F41" r:id="rId55" xr:uid="{0ECC354D-6B0E-48EA-86C1-FCB88AE23055}"/>
+    <hyperlink ref="I41" r:id="rId56" xr:uid="{E18A0679-D78E-4AD0-9AFB-C0AFE68021E3}"/>
+    <hyperlink ref="L41" r:id="rId57" xr:uid="{EA95F3A2-8876-4868-94D2-836712E7BF87}"/>
+    <hyperlink ref="O41" r:id="rId58" xr:uid="{32BBC9F7-6CFC-4E0E-A4FD-C361BEF34212}"/>
+    <hyperlink ref="R41" r:id="rId59" xr:uid="{3E48C8FE-C555-4326-B59D-077F6D0E6EE5}"/>
+    <hyperlink ref="F42" r:id="rId60" xr:uid="{4EB417D8-BA41-44F9-B1FD-969878DCC80F}"/>
+    <hyperlink ref="I42" r:id="rId61" xr:uid="{E6C977E9-9F9C-44AF-ADF7-E6D842301E29}"/>
+    <hyperlink ref="L42" r:id="rId62" xr:uid="{92A20403-229C-4590-A7D3-C53437FD757E}"/>
+    <hyperlink ref="O42" r:id="rId63" xr:uid="{DC9F8E70-901B-4B93-A393-AECDD229B4E1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId50"/>
+  <legacyDrawing r:id="rId64"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
N-ary tree BFS and binary tree algorithms and update progress tracking spreadsheet.
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FADB0A-7F9A-4842-856B-2F5FF2E54A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03830A8C-2DD8-44B3-BC6E-00AB6085D570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -191,7 +191,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="183">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -1837,14 +1837,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.31666666666666665</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -3536,7 +3536,7 @@
       <c r="W37" s="17"/>
       <c r="X37" s="17"/>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="10">
         <v>29</v>
       </c>
@@ -3550,7 +3550,9 @@
       <c r="D38" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E38" s="13"/>
+      <c r="E38" s="13">
+        <v>3</v>
+      </c>
       <c r="F38" s="31" t="s">
         <v>159</v>
       </c>
@@ -3607,7 +3609,7 @@
       </c>
       <c r="X38" s="16"/>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="10">
         <v>30</v>
       </c>
@@ -3621,7 +3623,9 @@
       <c r="D39" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E39" s="14"/>
+      <c r="E39" s="14">
+        <v>4</v>
+      </c>
       <c r="F39" s="32" t="s">
         <v>163</v>
       </c>
@@ -3634,7 +3638,9 @@
       <c r="I39" s="45" t="s">
         <v>164</v>
       </c>
-      <c r="J39" s="14"/>
+      <c r="J39" s="14" t="s">
+        <v>33</v>
+      </c>
       <c r="K39" s="14" t="s">
         <v>106</v>
       </c>
@@ -3674,18 +3680,23 @@
       </c>
       <c r="X39" s="17"/>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="10">
         <v>31</v>
       </c>
-      <c r="B40" s="23"/>
+      <c r="B40" s="23">
+        <f>B39+1</f>
+        <v>46191</v>
+      </c>
       <c r="C40" s="48" t="s">
         <v>72</v>
       </c>
       <c r="D40" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="E40" s="13"/>
+      <c r="E40" s="13">
+        <v>2</v>
+      </c>
       <c r="F40" s="32" t="str">
         <f>HYPERLINK("http://leetcode.com/problems/sum-root-to-leaf-numbers/","Sum Root to Leaf")</f>
         <v>Sum Root to Leaf</v>

</xml_diff>

<commit_message>
Heaps and Binary Search Tree operations
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA7B53D-7422-4109-AB55-788D12732157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E24F3BA-A369-459D-8E63-FA601F1D71EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -191,7 +191,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="187">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -741,9 +741,6 @@
     <t>Convert Sorted Array to BST</t>
   </si>
   <si>
-    <t>Minimum Absolute Difference in BST</t>
-  </si>
-  <si>
     <t>Two Sum IV - Input is a BST</t>
   </si>
   <si>
@@ -751,6 +748,21 @@
   </si>
   <si>
     <t>In Progress</t>
+  </si>
+  <si>
+    <t>Kth Largest Element in a Stream</t>
+  </si>
+  <si>
+    <t>Last Stone Weight</t>
+  </si>
+  <si>
+    <t>Relative Ranks</t>
+  </si>
+  <si>
+    <t>Take Gifts From the Richest Pile</t>
+  </si>
+  <si>
+    <t>Find Subsequence of Length K With the Largest Sum</t>
   </si>
 </sst>
 </file>
@@ -764,7 +776,7 @@
     <numFmt numFmtId="166" formatCode="dd/mmm/yyyy"/>
     <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -928,8 +940,21 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF467886"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1016,13 +1041,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF96ECB3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1056,7 +1087,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1167,11 +1198,19 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1428,6 +1467,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF96ECB3"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1759,6 +1803,9 @@
   <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </wetp:taskpane>
 </wetp:taskpanes>
 </file>
 
@@ -1770,6 +1817,20 @@
   </we:alternateReferences>
   <we:properties>
     <we:property name="claude.fileId" value="&quot;133bc33c-a07b-4139-8198-14c6b76d4ca5&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
+<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{3D43D1BF-0E5C-4C1E-96BB-B4524D28651F}">
+  <we:reference id="WA200010725" version="1.0.0.1" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="WA200010725" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;297a23cb-3c83-4ea5-a1b6-3bb65eff32cf&quot;"/>
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
@@ -1837,14 +1898,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.33333333333333331</v>
+        <v>0.35333333333333333</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1853,21 +1914,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.5499999999999998</v>
+        <v>2.5714285714285716</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="17" x14ac:dyDescent="0.4">
@@ -3544,7 +3605,7 @@
         <f>B32+3</f>
         <v>46189</v>
       </c>
-      <c r="C38" s="47" t="s">
+      <c r="C38" s="46" t="s">
         <v>69</v>
       </c>
       <c r="D38" s="13" t="s">
@@ -3617,7 +3678,7 @@
         <f>B38+1</f>
         <v>46190</v>
       </c>
-      <c r="C39" s="47" t="s">
+      <c r="C39" s="46" t="s">
         <v>70</v>
       </c>
       <c r="D39" s="14" t="s">
@@ -3688,7 +3749,7 @@
         <f>B39+1</f>
         <v>46191</v>
       </c>
-      <c r="C40" s="48" t="s">
+      <c r="C40" s="47" t="s">
         <v>72</v>
       </c>
       <c r="D40" s="13" t="s">
@@ -3739,7 +3800,7 @@
       </c>
       <c r="U40" s="13"/>
       <c r="V40" s="13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="W40" s="36">
         <v>1647433</v>
@@ -3754,7 +3815,7 @@
         <f>B40+1</f>
         <v>46192</v>
       </c>
-      <c r="C41" s="48" t="s">
+      <c r="C41" s="47" t="s">
         <v>73</v>
       </c>
       <c r="D41" s="14" t="s">
@@ -3803,7 +3864,9 @@
       <c r="R41" s="32" t="s">
         <v>177</v>
       </c>
-      <c r="S41" s="14"/>
+      <c r="S41" s="14" t="s">
+        <v>33</v>
+      </c>
       <c r="T41" s="14" t="s">
         <v>105</v>
       </c>
@@ -3823,81 +3886,125 @@
         <v>33</v>
       </c>
       <c r="B42" s="23">
-        <f>B41+1</f>
-        <v>46193</v>
-      </c>
-      <c r="C42" s="48" t="s">
+        <f>B41+2</f>
+        <v>46194</v>
+      </c>
+      <c r="C42" s="47" t="s">
         <v>74</v>
       </c>
       <c r="D42" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="E42" s="13"/>
+      <c r="E42" s="13">
+        <v>2</v>
+      </c>
       <c r="F42" s="31" t="s">
         <v>178</v>
       </c>
-      <c r="G42" s="13"/>
+      <c r="G42" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="H42" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="I42" s="31" t="s">
+      <c r="I42" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/kth-smallest-element-in-a-bst/description/","KthSmallestValueinBST")</f>
+        <v>KthSmallestValueinBST</v>
+      </c>
+      <c r="J42" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="K42" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L42" s="31" t="s">
         <v>179</v>
       </c>
-      <c r="J42" s="13"/>
-      <c r="K42" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="L42" s="31" t="s">
+      <c r="M42" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N42" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="O42" s="31" t="s">
         <v>180</v>
       </c>
-      <c r="M42" s="13"/>
-      <c r="N42" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="O42" s="31" t="s">
-        <v>181</v>
-      </c>
-      <c r="P42" s="13"/>
+      <c r="P42" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="Q42" s="13" t="s">
         <v>105</v>
       </c>
       <c r="R42" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="S42" s="13"/>
+      <c r="S42" s="13" t="s">
+        <v>35</v>
+      </c>
       <c r="T42" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="U42" s="13"/>
-      <c r="V42" s="13"/>
-      <c r="W42" s="16"/>
+      <c r="U42" s="13">
+        <v>3</v>
+      </c>
+      <c r="V42" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="W42" s="36">
+        <v>1523294</v>
+      </c>
       <c r="X42" s="16"/>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A43" s="10">
         <v>34</v>
       </c>
-      <c r="B43" s="23"/>
+      <c r="B43" s="23">
+        <f>B42+3</f>
+        <v>46197</v>
+      </c>
       <c r="C43" s="35" t="s">
         <v>75</v>
       </c>
-      <c r="D43" s="14"/>
+      <c r="D43" s="48" t="s">
+        <v>41</v>
+      </c>
       <c r="E43" s="14"/>
-      <c r="F43" s="12"/>
+      <c r="F43" s="49" t="s">
+        <v>182</v>
+      </c>
       <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="12"/>
+      <c r="H43" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="I43" s="49" t="s">
+        <v>183</v>
+      </c>
       <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
-      <c r="L43" s="12"/>
+      <c r="K43" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="L43" s="49" t="s">
+        <v>184</v>
+      </c>
       <c r="M43" s="14"/>
-      <c r="N43" s="14"/>
-      <c r="O43" s="12"/>
+      <c r="N43" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="O43" s="49" t="s">
+        <v>185</v>
+      </c>
       <c r="P43" s="14"/>
-      <c r="Q43" s="14"/>
-      <c r="R43" s="12"/>
+      <c r="Q43" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="R43" s="49" t="s">
+        <v>186</v>
+      </c>
       <c r="S43" s="14"/>
-      <c r="T43" s="14"/>
+      <c r="T43" s="48" t="s">
+        <v>106</v>
+      </c>
       <c r="U43" s="14"/>
       <c r="V43" s="14"/>
       <c r="W43" s="17"/>
@@ -3931,7 +4038,7 @@
       <c r="W44" s="16"/>
       <c r="X44" s="16"/>
     </row>
-    <row r="45" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A45" s="10">
         <v>36</v>
       </c>
@@ -3961,7 +4068,7 @@
       <c r="W45" s="17"/>
       <c r="X45" s="17"/>
     </row>
-    <row r="46" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A46" s="10">
         <v>37</v>
       </c>
@@ -3996,7 +4103,7 @@
         <v>38</v>
       </c>
       <c r="B47" s="23"/>
-      <c r="C47" s="46" t="s">
+      <c r="C47" s="52" t="s">
         <v>79</v>
       </c>
       <c r="D47" s="14"/>
@@ -4026,7 +4133,7 @@
         <v>39</v>
       </c>
       <c r="B48" s="23"/>
-      <c r="C48" s="46" t="s">
+      <c r="C48" s="52" t="s">
         <v>80</v>
       </c>
       <c r="D48" s="13"/>
@@ -4056,7 +4163,7 @@
         <v>40</v>
       </c>
       <c r="B49" s="23"/>
-      <c r="C49" s="46" t="s">
+      <c r="C49" s="52" t="s">
         <v>81</v>
       </c>
       <c r="D49" s="14"/>
@@ -4086,7 +4193,7 @@
         <v>41</v>
       </c>
       <c r="B50" s="23"/>
-      <c r="C50" s="46" t="s">
+      <c r="C50" s="52" t="s">
         <v>82</v>
       </c>
       <c r="D50" s="13"/>
@@ -4116,7 +4223,7 @@
         <v>42</v>
       </c>
       <c r="B51" s="23"/>
-      <c r="C51" s="46" t="s">
+      <c r="C51" s="52" t="s">
         <v>83</v>
       </c>
       <c r="D51" s="14"/>
@@ -4146,7 +4253,7 @@
         <v>43</v>
       </c>
       <c r="B52" s="23"/>
-      <c r="C52" s="46" t="s">
+      <c r="C52" s="52" t="s">
         <v>84</v>
       </c>
       <c r="D52" s="13"/>
@@ -4176,7 +4283,7 @@
         <v>44</v>
       </c>
       <c r="B53" s="23"/>
-      <c r="C53" s="46" t="s">
+      <c r="C53" s="52" t="s">
         <v>85</v>
       </c>
       <c r="D53" s="14"/>
@@ -4206,7 +4313,7 @@
         <v>45</v>
       </c>
       <c r="B54" s="23"/>
-      <c r="C54" s="46" t="s">
+      <c r="C54" s="52" t="s">
         <v>86</v>
       </c>
       <c r="D54" s="13"/>
@@ -4235,8 +4342,11 @@
       <c r="A55" s="10">
         <v>46</v>
       </c>
-      <c r="B55" s="23"/>
-      <c r="C55" s="35" t="s">
+      <c r="B55" s="23">
+        <f>B43+3</f>
+        <v>46200</v>
+      </c>
+      <c r="C55" s="50" t="s">
         <v>87</v>
       </c>
       <c r="D55" s="14"/>
@@ -4266,7 +4376,7 @@
         <v>47</v>
       </c>
       <c r="B56" s="23"/>
-      <c r="C56" s="35" t="s">
+      <c r="C56" s="50" t="s">
         <v>88</v>
       </c>
       <c r="D56" s="13"/>
@@ -4296,7 +4406,7 @@
         <v>48</v>
       </c>
       <c r="B57" s="23"/>
-      <c r="C57" s="35" t="s">
+      <c r="C57" s="50" t="s">
         <v>89</v>
       </c>
       <c r="D57" s="14"/>
@@ -4326,7 +4436,7 @@
         <v>49</v>
       </c>
       <c r="B58" s="23"/>
-      <c r="C58" s="35" t="s">
+      <c r="C58" s="50" t="s">
         <v>90</v>
       </c>
       <c r="D58" s="13"/>
@@ -4356,7 +4466,7 @@
         <v>50</v>
       </c>
       <c r="B59" s="23"/>
-      <c r="C59" s="35" t="s">
+      <c r="C59" s="50" t="s">
         <v>91</v>
       </c>
       <c r="D59" s="14"/>
@@ -4386,7 +4496,7 @@
         <v>51</v>
       </c>
       <c r="B60" s="23"/>
-      <c r="C60" s="35" t="s">
+      <c r="C60" s="50" t="s">
         <v>92</v>
       </c>
       <c r="D60" s="13"/>
@@ -4416,7 +4526,7 @@
         <v>52</v>
       </c>
       <c r="B61" s="23"/>
-      <c r="C61" s="35" t="s">
+      <c r="C61" s="50" t="s">
         <v>93</v>
       </c>
       <c r="D61" s="14"/>
@@ -4446,7 +4556,7 @@
         <v>53</v>
       </c>
       <c r="B62" s="23"/>
-      <c r="C62" s="35" t="s">
+      <c r="C62" s="50" t="s">
         <v>94</v>
       </c>
       <c r="D62" s="13"/>
@@ -4476,7 +4586,7 @@
         <v>54</v>
       </c>
       <c r="B63" s="23"/>
-      <c r="C63" s="35" t="s">
+      <c r="C63" s="50" t="s">
         <v>95</v>
       </c>
       <c r="D63" s="14"/>
@@ -4506,7 +4616,7 @@
         <v>55</v>
       </c>
       <c r="B64" s="23"/>
-      <c r="C64" s="15" t="s">
+      <c r="C64" s="51" t="s">
         <v>96</v>
       </c>
       <c r="D64" s="13"/>
@@ -4536,7 +4646,7 @@
         <v>56</v>
       </c>
       <c r="B65" s="23"/>
-      <c r="C65" s="15" t="s">
+      <c r="C65" s="51" t="s">
         <v>97</v>
       </c>
       <c r="D65" s="14"/>
@@ -4891,11 +5001,16 @@
     <hyperlink ref="O41" r:id="rId58" xr:uid="{32BBC9F7-6CFC-4E0E-A4FD-C361BEF34212}"/>
     <hyperlink ref="R41" r:id="rId59" xr:uid="{3E48C8FE-C555-4326-B59D-077F6D0E6EE5}"/>
     <hyperlink ref="F42" r:id="rId60" xr:uid="{4EB417D8-BA41-44F9-B1FD-969878DCC80F}"/>
-    <hyperlink ref="I42" r:id="rId61" xr:uid="{E6C977E9-9F9C-44AF-ADF7-E6D842301E29}"/>
+    <hyperlink ref="I42" r:id="rId61" display="Minimum Absolute Difference in BST" xr:uid="{E6C977E9-9F9C-44AF-ADF7-E6D842301E29}"/>
     <hyperlink ref="L42" r:id="rId62" xr:uid="{92A20403-229C-4590-A7D3-C53437FD757E}"/>
     <hyperlink ref="O42" r:id="rId63" xr:uid="{DC9F8E70-901B-4B93-A393-AECDD229B4E1}"/>
+    <hyperlink ref="F43" r:id="rId64" tooltip="Kth Largest Element in a Stream" xr:uid="{ACB876EA-47E0-485F-8495-FBB6BE6707EE}"/>
+    <hyperlink ref="I43" r:id="rId65" tooltip="Last Stone Weight" xr:uid="{4FA580D7-FD80-48A8-A10F-73014F5E35EE}"/>
+    <hyperlink ref="L43" r:id="rId66" tooltip="Relative Ranks" xr:uid="{454D593E-B1CD-495C-BDFF-7BB8051D8F80}"/>
+    <hyperlink ref="O43" r:id="rId67" tooltip="Take Gifts From the Richest Pile" xr:uid="{ED1BDAB4-926B-4A04-985F-7BE506D6D323}"/>
+    <hyperlink ref="R43" r:id="rId68" tooltip="Find Subsequence of Length K With the Largest Sum" xr:uid="{F6DD1F64-D233-496F-8266-0DDCF323AFC6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId64"/>
+  <legacyDrawing r:id="rId69"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dynamic programming study notes and implementations for 1D and 2D problems
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E24F3BA-A369-459D-8E63-FA601F1D71EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7F61A0-6B4C-41CC-BCE9-EC0C5F51E8C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -191,7 +192,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="192">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -763,6 +764,21 @@
   </si>
   <si>
     <t>Find Subsequence of Length K With the Largest Sum</t>
+  </si>
+  <si>
+    <t>Min Cost Climbing Stairs</t>
+  </si>
+  <si>
+    <t>Pascal's Triangle</t>
+  </si>
+  <si>
+    <t>Pascal's Triangle II</t>
+  </si>
+  <si>
+    <t>Counting Bits</t>
+  </si>
+  <si>
+    <t>Range Sum Query - Immutable</t>
   </si>
 </sst>
 </file>
@@ -1803,7 +1819,7 @@
   <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="525" row="2">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1898,14 +1914,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.35333333333333333</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1914,21 +1930,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.5714285714285716</v>
+        <v>2.5909090909090908</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="17" x14ac:dyDescent="0.4">
@@ -4038,7 +4054,7 @@
       <c r="W44" s="16"/>
       <c r="X44" s="16"/>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="10">
         <v>36</v>
       </c>
@@ -4068,7 +4084,7 @@
       <c r="W45" s="17"/>
       <c r="X45" s="17"/>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="10">
         <v>37</v>
       </c>
@@ -4098,7 +4114,7 @@
       <c r="W46" s="16"/>
       <c r="X46" s="16"/>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10">
         <v>38</v>
       </c>
@@ -4128,7 +4144,7 @@
       <c r="W47" s="17"/>
       <c r="X47" s="17"/>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="10">
         <v>39</v>
       </c>
@@ -4158,7 +4174,7 @@
       <c r="W48" s="16"/>
       <c r="X48" s="16"/>
     </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="10">
         <v>40</v>
       </c>
@@ -4188,7 +4204,7 @@
       <c r="W49" s="17"/>
       <c r="X49" s="17"/>
     </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="10">
         <v>41</v>
       </c>
@@ -4218,7 +4234,7 @@
       <c r="W50" s="16"/>
       <c r="X50" s="16"/>
     </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10">
         <v>42</v>
       </c>
@@ -4248,7 +4264,7 @@
       <c r="W51" s="17"/>
       <c r="X51" s="17"/>
     </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="10">
         <v>43</v>
       </c>
@@ -4278,7 +4294,7 @@
       <c r="W52" s="16"/>
       <c r="X52" s="16"/>
     </row>
-    <row r="53" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="10">
         <v>44</v>
       </c>
@@ -4308,7 +4324,7 @@
       <c r="W53" s="17"/>
       <c r="X53" s="17"/>
     </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="10">
         <v>45</v>
       </c>
@@ -4349,53 +4365,123 @@
       <c r="C55" s="50" t="s">
         <v>87</v>
       </c>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="12"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="12"/>
-      <c r="J55" s="14"/>
-      <c r="K55" s="14"/>
-      <c r="L55" s="12"/>
-      <c r="M55" s="14"/>
-      <c r="N55" s="14"/>
-      <c r="O55" s="12"/>
-      <c r="P55" s="14"/>
-      <c r="Q55" s="14"/>
-      <c r="R55" s="12"/>
-      <c r="S55" s="14"/>
-      <c r="T55" s="14"/>
-      <c r="U55" s="14"/>
-      <c r="V55" s="14"/>
-      <c r="W55" s="17"/>
+      <c r="D55" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E55" s="14">
+        <v>4</v>
+      </c>
+      <c r="F55" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/climbing-stairs/description/", "Climbing Stairs")</f>
+        <v>Climbing Stairs</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="H55" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="I55" s="32" t="str">
+        <f>HYPERLINK("https://www.geeksforgeeks.org/problems/geek-jump/1", "Frog Jump")</f>
+        <v>Frog Jump</v>
+      </c>
+      <c r="J55" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="K55" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="L55" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/house-robber/", "House Robber")</f>
+        <v>House Robber</v>
+      </c>
+      <c r="M55" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="N55" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="O55" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/unique-paths/", "Unique Paths")</f>
+        <v>Unique Paths</v>
+      </c>
+      <c r="P55" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q55" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="R55" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/minimum-path-sum/description/", "Minimum Path Sum")</f>
+        <v>Minimum Path Sum</v>
+      </c>
+      <c r="S55" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="T55" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="U55" s="14">
+        <v>3</v>
+      </c>
+      <c r="V55" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="W55" s="41">
+        <v>1456911</v>
+      </c>
       <c r="X55" s="17"/>
     </row>
     <row r="56" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A56" s="10">
         <v>47</v>
       </c>
-      <c r="B56" s="23"/>
+      <c r="B56" s="23">
+        <f>B55+3</f>
+        <v>46203</v>
+      </c>
       <c r="C56" s="50" t="s">
         <v>88</v>
       </c>
-      <c r="D56" s="13"/>
+      <c r="D56" s="48" t="s">
+        <v>41</v>
+      </c>
       <c r="E56" s="13"/>
-      <c r="F56" s="11"/>
+      <c r="F56" s="49" t="s">
+        <v>187</v>
+      </c>
       <c r="G56" s="13"/>
-      <c r="H56" s="13"/>
-      <c r="I56" s="11"/>
+      <c r="H56" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="I56" s="49" t="s">
+        <v>188</v>
+      </c>
       <c r="J56" s="13"/>
-      <c r="K56" s="13"/>
-      <c r="L56" s="11"/>
+      <c r="K56" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="L56" s="49" t="s">
+        <v>189</v>
+      </c>
       <c r="M56" s="13"/>
-      <c r="N56" s="13"/>
-      <c r="O56" s="11"/>
+      <c r="N56" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="O56" s="49" t="s">
+        <v>190</v>
+      </c>
       <c r="P56" s="13"/>
-      <c r="Q56" s="13"/>
-      <c r="R56" s="11"/>
+      <c r="Q56" s="48" t="s">
+        <v>106</v>
+      </c>
+      <c r="R56" s="49" t="s">
+        <v>191</v>
+      </c>
       <c r="S56" s="13"/>
-      <c r="T56" s="13"/>
+      <c r="T56" s="48" t="s">
+        <v>106</v>
+      </c>
       <c r="U56" s="13"/>
       <c r="V56" s="13"/>
       <c r="W56" s="16"/>
@@ -5009,8 +5095,16 @@
     <hyperlink ref="L43" r:id="rId66" tooltip="Relative Ranks" xr:uid="{454D593E-B1CD-495C-BDFF-7BB8051D8F80}"/>
     <hyperlink ref="O43" r:id="rId67" tooltip="Take Gifts From the Richest Pile" xr:uid="{ED1BDAB4-926B-4A04-985F-7BE506D6D323}"/>
     <hyperlink ref="R43" r:id="rId68" tooltip="Find Subsequence of Length K With the Largest Sum" xr:uid="{F6DD1F64-D233-496F-8266-0DDCF323AFC6}"/>
+    <hyperlink ref="O55" r:id="rId69" tooltip="Fibonacci Number" display="Fibonacci Number" xr:uid="{C9871103-54C8-4DBC-ABF6-87F012E33D42}"/>
+    <hyperlink ref="R55" r:id="rId70" tooltip="N-th Tribonacci Number" display="N-th Tribonacci Number" xr:uid="{3F0EA806-31A3-440A-83F2-9AF5C851AA9E}"/>
+    <hyperlink ref="F56" r:id="rId71" tooltip="Min Cost Climbing Stairs" xr:uid="{E4E6A500-AA07-4E6D-AF43-7BC85E392D5D}"/>
+    <hyperlink ref="I56" r:id="rId72" tooltip="Pascal's Triangle" xr:uid="{CBEFACE6-E614-45F1-964F-7CAD737FF17E}"/>
+    <hyperlink ref="L56" r:id="rId73" tooltip="Pascal's Triangle II" xr:uid="{091D8C20-1BAA-485C-85F9-7C5335211BA3}"/>
+    <hyperlink ref="O56" r:id="rId74" tooltip="Counting Bits" xr:uid="{059A599F-CA30-44F4-92C5-D64DD9509163}"/>
+    <hyperlink ref="R56" r:id="rId75" tooltip="Range Sum Query - Immutable" xr:uid="{B42D7F33-7400-48DD-9B7B-E859B1E17C1F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId69"/>
+  <pageSetup orientation="portrait" r:id="rId76"/>
+  <legacyDrawing r:id="rId77"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Greedy algorithm problems including Interval Scheduling, Fractional Knapsack, and Meeting Rooms
</commit_message>
<xml_diff>
--- a/DSA Practice.xlsx
+++ b/DSA Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dushyant\Desktop\DSA Practice\Data-Structures-Algorithms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7F61A0-6B4C-41CC-BCE9-EC0C5F51E8C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBDB9099-7FF3-4D5D-BB89-A0CCDBA83394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{11A40645-F60E-40B0-9503-F1433C5B797F}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -192,7 +191,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="194">
   <si>
     <t>Quick Stats</t>
   </si>
@@ -779,6 +778,12 @@
   </si>
   <si>
     <t>Range Sum Query - Immutable</t>
+  </si>
+  <si>
+    <t>Meeting Rooms</t>
+  </si>
+  <si>
+    <t>Can Place Flowers</t>
   </si>
 </sst>
 </file>
@@ -1914,14 +1919,14 @@
       </c>
       <c r="D5" s="5" cm="1">
         <f t="array" ref="D5">SUMPRODUCT((G10:G69&lt;&gt;"")*1)+SUMPRODUCT((J10:J69&lt;&gt;"")*1)+SUMPRODUCT((M10:M69&lt;&gt;"")*1)+SUMPRODUCT((P10:P69&lt;&gt;"")*1)+SUMPRODUCT((S10:S69&lt;&gt;"")*1)</f>
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6">
         <f>D5/B5</f>
-        <v>0.37</v>
+        <v>0.38666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="22" customFormat="1" x14ac:dyDescent="0.35">
@@ -1930,21 +1935,21 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(V10:V69,"Done")</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="7">
         <f>60-B6</f>
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>IFERROR(AVERAGE(U10:U69),0)</f>
-        <v>2.5909090909090908</v>
+        <v>2.6086956521739131</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="17" x14ac:dyDescent="0.4">
@@ -4701,30 +4706,66 @@
       <c r="A64" s="10">
         <v>55</v>
       </c>
-      <c r="B64" s="23"/>
+      <c r="B64" s="23">
+        <f>B56+2</f>
+        <v>46205</v>
+      </c>
       <c r="C64" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D64" s="13"/>
-      <c r="E64" s="13"/>
-      <c r="F64" s="11"/>
-      <c r="G64" s="13"/>
+      <c r="D64" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E64" s="13">
+        <v>3</v>
+      </c>
+      <c r="F64" s="31" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/assign-cookies/description/","Assign Cookies")</f>
+        <v>Assign Cookies</v>
+      </c>
+      <c r="G64" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="H64" s="13"/>
-      <c r="I64" s="11"/>
+      <c r="I64" s="31" t="s">
+        <v>192</v>
+      </c>
       <c r="J64" s="13"/>
-      <c r="K64" s="13"/>
-      <c r="L64" s="11"/>
-      <c r="M64" s="13"/>
+      <c r="K64" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L64" s="31" t="str">
+        <f>HYPERLINK("https://www.geeksforgeeks.org/problems/fractional-knapsack-1587115620/1","Fractional Knapsack")</f>
+        <v>Fractional Knapsack</v>
+      </c>
+      <c r="M64" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="N64" s="13"/>
-      <c r="O64" s="11"/>
+      <c r="O64" s="31" t="s">
+        <v>193</v>
+      </c>
       <c r="P64" s="13"/>
-      <c r="Q64" s="13"/>
-      <c r="R64" s="11"/>
-      <c r="S64" s="13"/>
+      <c r="Q64" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="R64" s="31" t="str">
+        <f>HYPERLINK("#https://www.geeksforgeeks.org/problems/-minimum-number-of-coins4426/1","Minimum No of Coins")</f>
+        <v>Minimum No of Coins</v>
+      </c>
+      <c r="S64" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="T64" s="13"/>
-      <c r="U64" s="13"/>
-      <c r="V64" s="13"/>
-      <c r="W64" s="16"/>
+      <c r="U64" s="13">
+        <v>3</v>
+      </c>
+      <c r="V64" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="W64" s="36">
+        <v>1426671</v>
+      </c>
       <c r="X64" s="16"/>
     </row>
     <row r="65" spans="1:24" x14ac:dyDescent="0.35">
@@ -4737,11 +4778,21 @@
       </c>
       <c r="D65" s="14"/>
       <c r="E65" s="14"/>
-      <c r="F65" s="12"/>
-      <c r="G65" s="14"/>
+      <c r="F65" s="32" t="str">
+        <f>HYPERLINK("https://leetcode.com/problems/lemonade-change/description/","Lemonade Change")</f>
+        <v>Lemonade Change</v>
+      </c>
+      <c r="G65" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="H65" s="14"/>
-      <c r="I65" s="12"/>
-      <c r="J65" s="14"/>
+      <c r="I65" s="32" t="str">
+        <f>HYPERLINK("https://www.geeksforgeeks.org/problems/activity-selection-1587115620/1","Max Meetings")</f>
+        <v>Max Meetings</v>
+      </c>
+      <c r="J65" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="K65" s="14"/>
       <c r="L65" s="12"/>
       <c r="M65" s="14"/>
@@ -4754,7 +4805,9 @@
       <c r="T65" s="14"/>
       <c r="U65" s="14"/>
       <c r="V65" s="14"/>
-      <c r="W65" s="17"/>
+      <c r="W65" s="41">
+        <v>1407317</v>
+      </c>
       <c r="X65" s="17"/>
     </row>
     <row r="66" spans="1:24" x14ac:dyDescent="0.35">
@@ -5102,9 +5155,11 @@
     <hyperlink ref="L56" r:id="rId73" tooltip="Pascal's Triangle II" xr:uid="{091D8C20-1BAA-485C-85F9-7C5335211BA3}"/>
     <hyperlink ref="O56" r:id="rId74" tooltip="Counting Bits" xr:uid="{059A599F-CA30-44F4-92C5-D64DD9509163}"/>
     <hyperlink ref="R56" r:id="rId75" tooltip="Range Sum Query - Immutable" xr:uid="{B42D7F33-7400-48DD-9B7B-E859B1E17C1F}"/>
+    <hyperlink ref="I64" r:id="rId76" tooltip="Open on LeetCode" xr:uid="{D9D9E246-1101-44A0-A54B-009650EC2006}"/>
+    <hyperlink ref="O64" r:id="rId77" tooltip="Open on LeetCode" xr:uid="{133AEADC-BC51-4AB2-B8E4-DBA8DE0A1BE8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId76"/>
-  <legacyDrawing r:id="rId77"/>
+  <pageSetup orientation="portrait" r:id="rId78"/>
+  <legacyDrawing r:id="rId79"/>
 </worksheet>
 </file>
</xml_diff>